<commit_message>
feat: scripts SQL de creación, pruebas de restricciones y public_id (HU-03)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="237">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -161,10 +161,10 @@
     <t xml:space="preserve">11 entidades; cardinalidades y participación indicadas; estado del asiento por partido modelado</t>
   </si>
   <si>
-    <t xml:space="preserve">docs/HU-02-modelo-er · PR #1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 tablas en 3 BD. Pendiente: mover la carpeta a docs/modelo-er (quedó en docs-modelo-er/docs/...).</t>
+    <t xml:space="preserve">docs/HU-02-modelo-er · PR #1 · fix/HU-02-ruta-docs · PR #2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 tablas en 3 BD. Ruta corregida en PR #2. Actualizado con public_id UUID (decisión 12) en la rama de HU-03.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-03</t>
@@ -173,18 +173,27 @@
     <t xml:space="preserve">Como equipo, quiero un script SQL de creación con PK, FK y restricciones para generar la base de datos</t>
   </si>
   <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El script corre sin errores en una BD vacía; UNIQUE(partido, asiento); CHECK de tipos de sección</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-03-script-sql</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 scripts de esquema + 65 pruebas de restricciones (65/65 PASS en PostgreSQL 16). Incluye id interno BIGINT + public_id UUID. Falta commit y PR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero un script semilla con al menos 5 registros por tabla para tener datos de prueba</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">El script corre sin errores en una BD vacía; UNIQUE(partido, asiento); CHECK de tipos de sección</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero un script semilla con al menos 5 registros por tabla para tener datos de prueba</t>
-  </si>
-  <si>
     <t xml:space="preserve">≥5 registros por tabla; ninguna violación de FK ni de restricciones</t>
   </si>
   <si>
@@ -195,9 +204,6 @@
   </si>
   <si>
     <t xml:space="preserve">Repositorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En curso</t>
   </si>
   <si>
     <t xml:space="preserve">Entregable GitHub</t>
@@ -1471,11 +1477,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="58859689"/>
-        <c:axId val="76954000"/>
+        <c:axId val="81337084"/>
+        <c:axId val="36347730"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="58859689"/>
+        <c:axId val="81337084"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1541,7 +1547,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76954000"/>
+        <c:crossAx val="36347730"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1549,7 +1555,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76954000"/>
+        <c:axId val="36347730"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1625,7 +1631,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58859689"/>
+        <c:crossAx val="81337084"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2166,7 +2172,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
         <v>46</v>
       </c>
@@ -2198,15 +2204,19 @@
       <c r="K7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
+      <c r="L7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>31</v>
@@ -2224,30 +2234,30 @@
         <v>34</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I8" s="14"/>
       <c r="J8" s="5" t="s">
         <v>42</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>33</v>
@@ -2259,34 +2269,34 @@
         <v>34</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>36</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>33</v>
@@ -2295,33 +2305,33 @@
         <v>3</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>33</v>
@@ -2330,33 +2340,33 @@
         <v>5</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>33</v>
@@ -2365,33 +2375,33 @@
         <v>3</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>33</v>
@@ -2400,33 +2410,33 @@
         <v>3</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2435,33 +2445,33 @@
         <v>5</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2470,33 +2480,33 @@
         <v>5</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2505,33 +2515,33 @@
         <v>3</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2540,33 +2550,33 @@
         <v>2</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2575,33 +2585,33 @@
         <v>1</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2610,33 +2620,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2645,33 +2655,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2680,33 +2690,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2715,33 +2725,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2750,33 +2760,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2785,33 +2795,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2820,33 +2830,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2855,33 +2865,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2890,33 +2900,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2925,33 +2935,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -2960,33 +2970,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -2995,33 +3005,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3030,33 +3040,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3065,33 +3075,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3100,68 +3110,68 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>33</v>
@@ -3170,33 +3180,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3205,122 +3215,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>159</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>157</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3383,12 +3393,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3396,34 +3406,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3431,7 +3441,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3440,7 +3450,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3463,10 +3473,10 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3475,7 +3485,7 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3498,10 +3508,10 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3510,7 +3520,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3533,10 +3543,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3545,7 +3555,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3568,10 +3578,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3580,7 +3590,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3603,7 +3613,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3649,171 +3659,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3822,7 +3832,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3831,7 +3841,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3863,23 +3873,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat: datos semilla, verificaciones y script de setup (HU-04)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="241">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -173,63 +173,69 @@
     <t xml:space="preserve">Como equipo, quiero un script SQL de creación con PK, FK y restricciones para generar la base de datos</t>
   </si>
   <si>
+    <t xml:space="preserve">El script corre sin errores en una BD vacía; UNIQUE(partido, asiento); CHECK de tipos de sección</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-03-script-sql · PR #3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 scripts de esquema + 65 pruebas de restricciones (65/65 PASS). Id interno BIGINT + public_id UUID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero un script semilla con al menos 5 registros por tabla para tener datos de prueba</t>
+  </si>
+  <si>
     <t xml:space="preserve">En curso</t>
   </si>
   <si>
-    <t xml:space="preserve">El script corre sin errores en una BD vacía; UNIQUE(partido, asiento); CHECK de tipos de sección</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feature/HU-03-script-sql</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 scripts de esquema + 65 pruebas de restricciones (65/65 PASS en PostgreSQL 16). Incluye id interno BIGINT + public_id UUID. Falta commit y PR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero un script semilla con al menos 5 registros por tabla para tener datos de prueba</t>
+    <t xml:space="preserve">≥5 registros por tabla; ninguna violación de FK ni de restricciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-04-datos-semilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semillas de las 3 bases (≥5 por tabla, 610 asientos generados) + 36 verificaciones + setup-db.ps1. Se agregó el estado BLOQUEADO a app_user (106/106 PASS). Falta commit y PR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero un repositorio GitHub con carpetas backend y frontend para versionar el proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repositorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entregable GitHub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo creado con estructura backend/ y frontend/ y primer commit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo creado y primer PR integrado. Faltan carpetas backend/ y frontend/.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero registrar un escenario deportivo (nombre, descripción, ubicación, capacidad) para gestionar estadios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS Partidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 1</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">≥5 registros por tabla; ninguna violación de FK ni de restricciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero un repositorio GitHub con carpetas backend y frontend para versionar el proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repositorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entregable GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo creado con estructura backend/ y frontend/ y primer commit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo creado y primer PR integrado. Faltan carpetas backend/ y frontend/.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero registrar un escenario deportivo (nombre, descripción, ubicación, capacidad) para gestionar estadios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Funcional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS Partidos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Microservicio de partidos (5)</t>
   </si>
   <si>
@@ -287,7 +293,7 @@
     <t xml:space="preserve">Como usuario, quiero iniciar sesión y obtener un token según mi rol para acceder a mis funcionalidades</t>
   </si>
   <si>
-    <t xml:space="preserve">Credenciales malas → 401; usuario inactivo → 403; token con rol y expiración</t>
+    <t xml:space="preserve">Credenciales malas → 401 con mensaje genérico; usuario inactivo → 403; 5 intentos fallidos → BLOQUEADO 15 min (423); login exitoso reinicia el contador; token con rol y expiración</t>
   </si>
   <si>
     <t xml:space="preserve">HU-12</t>
@@ -609,6 +615,14 @@
   </si>
   <si>
     <t xml:space="preserve">Entorno instalado, modelo ER, script SQL de creación y semillas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incremento: modelo ER (12 tablas, 3 BD), scripts SQL con restricciones nombradas, datos semilla (≥5 por tabla) y setup-db.ps1. 106/106 pruebas PASS. La base ya soporta autenticación y autorización; la auditoría queda pendiente para el Sprint 2. HU-05 pasa al Sprint 1 (faltan carpetas backend/ y frontend/).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salió bien: crear las bases de datos y encontrar las relaciones entre las tablas.
+Costó: recordar el modelo entidad-relación y saber dónde va la FK.
+Acción de mejora: probar en Apidog cada endpoint apenas esté listo, no al final del sprint.</t>
   </si>
   <si>
     <t xml:space="preserve">Microservicios Partidos y Usuarios/Auth</t>
@@ -1435,34 +1449,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>116</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1477,11 +1491,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="81337084"/>
-        <c:axId val="36347730"/>
+        <c:axId val="66069689"/>
+        <c:axId val="65728187"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="81337084"/>
+        <c:axId val="66069689"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1547,7 +1561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36347730"/>
+        <c:crossAx val="65728187"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1555,7 +1569,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36347730"/>
+        <c:axId val="65728187"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1631,7 +1645,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81337084"/>
+        <c:crossAx val="66069689"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1959,7 +1973,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1968,7 +1982,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.0569105691056911</v>
+        <v>0.0813008130081301</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,7 +1991,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2172,7 +2186,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
         <v>46</v>
       </c>
@@ -2195,28 +2209,30 @@
         <v>34</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>46312</v>
+      </c>
       <c r="J7" s="5" t="s">
         <v>42</v>
       </c>
       <c r="K7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="15" t="s">
+      <c r="M7" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="M7" s="15" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="B8" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>31</v>
@@ -2234,30 +2250,34 @@
         <v>34</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" s="14"/>
       <c r="J8" s="5" t="s">
         <v>42</v>
       </c>
       <c r="K8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
+      <c r="M8" s="15" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>33</v>
@@ -2269,34 +2289,34 @@
         <v>34</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>36</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>33</v>
@@ -2305,33 +2325,33 @@
         <v>3</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>33</v>
@@ -2340,33 +2360,33 @@
         <v>5</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>33</v>
@@ -2375,33 +2395,33 @@
         <v>3</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>33</v>
@@ -2410,33 +2430,33 @@
         <v>3</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2445,33 +2465,33 @@
         <v>5</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2480,33 +2500,33 @@
         <v>5</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2515,33 +2535,33 @@
         <v>3</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2550,33 +2570,33 @@
         <v>2</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2585,33 +2605,33 @@
         <v>1</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2620,33 +2640,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2655,33 +2675,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2690,33 +2710,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2725,33 +2745,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2760,33 +2780,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2795,33 +2815,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2830,33 +2850,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2865,33 +2885,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2900,33 +2920,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2935,33 +2955,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -2970,33 +2990,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3005,33 +3025,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3040,33 +3060,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3075,33 +3095,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3110,68 +3130,68 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>33</v>
@@ -3180,33 +3200,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3215,122 +3235,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>161</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>159</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3393,12 +3413,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3406,42 +3426,42 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3450,7 +3470,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3462,21 +3482,25 @@
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A5,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">IF(G5=0,0,H5/G5)</f>
-        <v>0.5</v>
-      </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
+        <v>0.714285714285714</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3485,7 +3509,7 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3508,10 +3532,10 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3520,7 +3544,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3543,10 +3567,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3555,7 +3579,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3578,10 +3602,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3590,7 +3614,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3613,7 +3637,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3625,11 +3649,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.0569105691056911</v>
+        <v>0.0813008130081301</v>
       </c>
     </row>
   </sheetData>
@@ -3659,171 +3683,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3832,7 +3856,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3841,7 +3865,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3873,23 +3897,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3902,7 +3926,7 @@
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A5)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3915,7 +3939,7 @@
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A6)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3928,7 +3952,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3941,7 +3965,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3954,7 +3978,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3967,7 +3991,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3980,7 +4004,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3993,7 +4017,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4006,7 +4030,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4019,7 +4043,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: cierre del Sprint 0 y contrato con versión v1
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="243">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -188,34 +188,37 @@
     <t xml:space="preserve">Como equipo, quiero un script semilla con al menos 5 registros por tabla para tener datos de prueba</t>
   </si>
   <si>
+    <t xml:space="preserve">≥5 registros por tabla; ninguna violación de FK ni de restricciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-04-datos-semilla · PR #4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semillas de las 3 bases (≥5 por tabla, 610 asientos generados) + 36 verificaciones + setup-db.ps1 + estado BLOQUEADO. 106/106 PASS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero un repositorio GitHub con carpetas backend y frontend para versionar el proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repositorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">En curso</t>
   </si>
   <si>
-    <t xml:space="preserve">≥5 registros por tabla; ninguna violación de FK ni de restricciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feature/HU-04-datos-semilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semillas de las 3 bases (≥5 por tabla, 610 asientos generados) + 36 verificaciones + setup-db.ps1. Se agregó el estado BLOQUEADO a app_user (106/106 PASS). Falta commit y PR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero un repositorio GitHub con carpetas backend y frontend para versionar el proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repositorio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Entregable GitHub</t>
   </si>
   <si>
     <t xml:space="preserve">Repo creado con estructura backend/ y frontend/ y primer commit</t>
   </si>
   <si>
-    <t xml:space="preserve">Repo creado y primer PR integrado. Faltan carpetas backend/ y frontend/.</t>
+    <t xml:space="preserve">Repo con docs/ y database/ (PR #1–#4). Movida al Sprint 1: faltan backend/ y frontend/, que se crean con el primer microservicio.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-06</t>
@@ -230,24 +233,27 @@
     <t xml:space="preserve">MS Partidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 1</t>
+    <t xml:space="preserve">Microservicio de partidos (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRUD responde 201/200/404; capacidad positiva validada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/HU-06-contrato-ms-partidos · PR #5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato OpenAPI de ms-partidos (15 operaciones) en docs/apis/. Rutas /match-api/v1. Falta la implementación en Spring Boot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero registrar secciones (PALCOS, GENERAL, PREFERENCIA, TRIBUNAS), filas con letras y asientos para definir la distribución física</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Microservicio de partidos (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRUD responde 201/200/404; capacidad positiva validada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero registrar secciones (PALCOS, GENERAL, PREFERENCIA, TRIBUNAS), filas con letras y asientos para definir la distribución física</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tipo de sección fuera del catálogo → 400; filas A, B, C consecutivas; asientos generados por fila</t>
   </si>
   <si>
@@ -617,7 +623,7 @@
     <t xml:space="preserve">Entorno instalado, modelo ER, script SQL de creación y semillas</t>
   </si>
   <si>
-    <t xml:space="preserve">Incremento: modelo ER (12 tablas, 3 BD), scripts SQL con restricciones nombradas, datos semilla (≥5 por tabla) y setup-db.ps1. 106/106 pruebas PASS. La base ya soporta autenticación y autorización; la auditoría queda pendiente para el Sprint 2. HU-05 pasa al Sprint 1 (faltan carpetas backend/ y frontend/).</t>
+    <t xml:space="preserve">Incremento: modelo ER (12 tablas, 3 BD), scripts SQL con restricciones nombradas, datos semilla (≥5 por tabla) y setup-db.ps1. 106/106 pruebas PASS. La base ya soporta autenticación y autorización; la auditoría queda pendiente para el Sprint 2. HU-05 pasa al Sprint 1 (faltan carpetas backend/ y frontend/). Resumen completo en docs/sprints/sprint-0.md.</t>
   </si>
   <si>
     <t xml:space="preserve">Salió bien: crear las bases de datos y encontrar las relaciones entre las tablas.
@@ -1449,34 +1455,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>113</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1491,11 +1497,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="66069689"/>
-        <c:axId val="65728187"/>
+        <c:axId val="97502102"/>
+        <c:axId val="9445755"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="66069689"/>
+        <c:axId val="97502102"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1561,7 +1567,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65728187"/>
+        <c:crossAx val="9445755"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1569,7 +1575,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65728187"/>
+        <c:axId val="9445755"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1645,7 +1651,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66069689"/>
+        <c:crossAx val="97502102"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1973,7 +1979,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1982,7 +1988,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.0813008130081301</v>
+        <v>0.105691056910569</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1991,7 +1997,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2227,7 +2233,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>51</v>
       </c>
@@ -2250,34 +2256,36 @@
         <v>34</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>46312</v>
+      </c>
       <c r="J8" s="5" t="s">
         <v>42</v>
       </c>
       <c r="K8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="L8" s="15" t="s">
+      <c r="M8" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="M8" s="15" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>33</v>
@@ -2286,37 +2294,37 @@
         <v>1</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>36</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>33</v>
@@ -2325,33 +2333,37 @@
         <v>3</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="L10" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
+      <c r="M10" s="15" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>33</v>
@@ -2360,33 +2372,33 @@
         <v>5</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>33</v>
@@ -2395,33 +2407,33 @@
         <v>3</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>33</v>
@@ -2430,33 +2442,33 @@
         <v>3</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2465,33 +2477,33 @@
         <v>5</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2500,33 +2512,33 @@
         <v>5</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2535,33 +2547,33 @@
         <v>3</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2570,33 +2582,33 @@
         <v>2</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2605,33 +2617,33 @@
         <v>1</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2640,33 +2652,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2675,33 +2687,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2710,33 +2722,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2745,33 +2757,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2780,33 +2792,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2815,33 +2827,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2850,33 +2862,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2885,33 +2897,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2920,33 +2932,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2955,33 +2967,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -2990,33 +3002,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3025,33 +3037,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3060,33 +3072,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3095,33 +3107,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3130,68 +3142,68 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>33</v>
@@ -3200,33 +3212,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3235,122 +3247,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3413,12 +3425,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3426,42 +3438,42 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3470,37 +3482,37 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A5)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A5,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">IF(G5=0,0,H5/G5)</f>
-        <v>0.714285714285714</v>
+        <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3509,15 +3521,15 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
@@ -3532,10 +3544,10 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3544,7 +3556,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3567,10 +3579,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3579,7 +3591,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3602,10 +3614,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3614,7 +3626,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3637,7 +3649,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3649,11 +3661,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.0813008130081301</v>
+        <v>0.105691056910569</v>
       </c>
     </row>
   </sheetData>
@@ -3683,171 +3695,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3856,7 +3868,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3865,7 +3877,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3897,23 +3909,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3926,7 +3938,7 @@
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A5)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3939,7 +3951,7 @@
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A6)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3952,7 +3964,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3965,7 +3977,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3978,7 +3990,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3991,7 +4003,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4004,7 +4016,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,7 +4029,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4030,7 +4042,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4043,7 +4055,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(match-service): limitar capacidad a 200000 según contrato (HU-06)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="244">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -209,40 +209,43 @@
     <t xml:space="preserve">Sprint 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Entregable GitHub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo creado con estructura backend/ y frontend/ y primer commit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chore/HU-05-estructura-proyecto · PR #7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">backend/match-service (Spring Boot 4.1.1, Java 17, puerto 8082, conectado a match_db) y frontend/ (React + Vite, puerto 5173). Nombres en inglés: match-service, auth-service, reservation-service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero registrar un escenario deportivo (nombre, descripción, ubicación, capacidad) para gestionar estadios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS Partidos</t>
+  </si>
+  <si>
     <t xml:space="preserve">En curso</t>
   </si>
   <si>
-    <t xml:space="preserve">Entregable GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo creado con estructura backend/ y frontend/ y primer commit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo con docs/ y database/ (PR #1–#4). Movida al Sprint 1: faltan backend/ y frontend/, que se crean con el primer microservicio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero registrar un escenario deportivo (nombre, descripción, ubicación, capacidad) para gestionar estadios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Funcional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS Partidos</t>
-  </si>
-  <si>
     <t xml:space="preserve">Microservicio de partidos (5)</t>
   </si>
   <si>
     <t xml:space="preserve">CRUD responde 201/200/404; capacidad positiva validada</t>
   </si>
   <si>
-    <t xml:space="preserve">docs/HU-06-contrato-ms-partidos · PR #5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contrato OpenAPI de ms-partidos (15 operaciones) en docs/apis/. Rutas /match-api/v1. Falta la implementación en Spring Boot.</t>
+    <t xml:space="preserve">docs/HU-06-contrato-ms-partidos · PR #5 · feature/HU-06-crud-estadios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato OpenAPI (PR #5). Implementado: GET /stadiums (orden por id), GET /stadiums/{id} (404 Problem Details), POST /stadiums (201 + Location; 400 con errores por campo; 409 por nombre duplicado en 2 capas: servicio + uk_stadium_name; listas blancas con @Pattern contra inyección/XSS). Falta: PUT y DELETE. Riesgo abierto: match-service sin Spring Security hasta HU-11/12 (escritura expuesta). Mejora: uk_stadium_name distingue mayúsculas → índice único sobre LOWER(name).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-07</t>
@@ -1458,31 +1461,31 @@
                   <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>110</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1497,11 +1500,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="97502102"/>
-        <c:axId val="9445755"/>
+        <c:axId val="63702391"/>
+        <c:axId val="15645428"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="97502102"/>
+        <c:axId val="63702391"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1567,7 +1570,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9445755"/>
+        <c:crossAx val="15645428"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1575,7 +1578,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9445755"/>
+        <c:axId val="15645428"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1651,7 +1654,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97502102"/>
+        <c:crossAx val="63702391"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1979,7 +1982,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1988,7 +1991,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.105691056910569</v>
+        <v>0.113821138211382</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1997,7 +2000,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2274,7 +2277,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
         <v>56</v>
       </c>
@@ -2297,23 +2300,25 @@
         <v>59</v>
       </c>
       <c r="H9" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>46313</v>
+      </c>
+      <c r="J9" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="I9" s="14"/>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="15" t="s">
         <v>62</v>
-      </c>
-      <c r="L9" s="15" t="s">
-        <v>36</v>
       </c>
       <c r="M9" s="15" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>64</v>
       </c>
@@ -2336,28 +2341,28 @@
         <v>59</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>66</v>
@@ -2375,24 +2380,24 @@
         <v>59</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>66</v>
@@ -2410,24 +2415,24 @@
         <v>59</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>66</v>
@@ -2445,30 +2450,30 @@
         <v>59</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2480,30 +2485,30 @@
         <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2515,30 +2520,30 @@
         <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2550,30 +2555,30 @@
         <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2585,30 +2590,30 @@
         <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2620,30 +2625,30 @@
         <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2652,33 +2657,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2687,33 +2692,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2722,33 +2727,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2757,33 +2762,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2792,33 +2797,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2827,33 +2832,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2862,33 +2867,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2897,33 +2902,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2932,33 +2937,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2967,33 +2972,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3002,33 +3007,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3037,33 +3042,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3072,33 +3077,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3107,33 +3112,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3142,62 +3147,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3212,33 +3217,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3247,122 +3252,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3425,12 +3430,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3438,34 +3443,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,7 +3478,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3482,7 +3487,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3501,10 +3506,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3512,7 +3517,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3521,7 +3526,7 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3533,21 +3538,21 @@
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
-        <v>0</v>
+        <v>0.032258064516129</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3556,7 +3561,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3579,10 +3584,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3591,7 +3596,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3614,10 +3619,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3626,7 +3631,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3649,7 +3654,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3661,11 +3666,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.105691056910569</v>
+        <v>0.113821138211382</v>
       </c>
     </row>
   </sheetData>
@@ -3695,171 +3700,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3868,7 +3873,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3877,7 +3882,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3909,23 +3914,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3951,7 +3956,7 @@
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A6)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3964,7 +3969,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,7 +3982,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3990,7 +3995,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4003,7 +4008,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4016,7 +4021,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4029,7 +4034,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4042,7 +4047,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4055,7 +4060,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(match-service): crear y consultar partidos con validación de fecha (HU-08), feat(match-service): editar partido con máquina de estados (HU-08)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="245">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -251,16 +251,22 @@
     <t xml:space="preserve">Como administrador, quiero registrar secciones (PALCOS, GENERAL, PREFERENCIA, TRIBUNAS), filas con letras y asientos para definir la distribución física</t>
   </si>
   <si>
+    <t xml:space="preserve">Tipo de sección fuera del catálogo → 400; filas A, B, C consecutivas; asientos generados por fila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-07-secciones · PR #9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidades Section/SeatRow/Seat con relaciones y cascade. GET y POST de secciones: genera filas A..Z y asientos 1..N en una transacción. 400 tipo fuera de catálogo / rangos; 404; 409 nombre por estadio; 422 si supera la capacidad del estadio. Pendiente (nueva HU): editar/eliminar sección y endpoint layout. Mejora: bloqueo pesimista para la regla de capacidad con concurrencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero registrar partidos (nombre, descripción, fecha, hora, estado, escenario) para publicarlos</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de sección fuera del catálogo → 400; filas A, B, C consecutivas; asientos generados por fila</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero registrar partidos (nombre, descripción, fecha, hora, estado, escenario) para publicarlos</t>
   </si>
   <si>
     <t xml:space="preserve">Escenario inexistente → 404; fecha pasada rechazada</t>
@@ -1450,31 +1456,31 @@
                   <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>106</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1489,11 +1495,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="54093656"/>
-        <c:axId val="57014940"/>
+        <c:axId val="51158772"/>
+        <c:axId val="42992183"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="54093656"/>
+        <c:axId val="51158772"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1559,7 +1565,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57014940"/>
+        <c:crossAx val="42992183"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1567,7 +1573,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57014940"/>
+        <c:axId val="42992183"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1643,7 +1649,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54093656"/>
+        <c:crossAx val="51158772"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1971,7 +1977,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1980,7 +1986,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.138211382113821</v>
+        <v>0.178861788617886</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1989,7 +1995,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2348,7 +2354,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
         <v>72</v>
       </c>
@@ -2371,24 +2377,30 @@
         <v>59</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="I11" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>46313</v>
+      </c>
       <c r="J11" s="5" t="s">
         <v>68</v>
       </c>
       <c r="K11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="L11" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
+      <c r="M11" s="15" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>66</v>
@@ -2406,24 +2418,24 @@
         <v>59</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="5" t="s">
         <v>68</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>66</v>
@@ -2441,30 +2453,30 @@
         <v>59</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2476,30 +2488,30 @@
         <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2511,30 +2523,30 @@
         <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2546,30 +2558,30 @@
         <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2581,30 +2593,30 @@
         <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2616,30 +2628,30 @@
         <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2648,33 +2660,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2683,33 +2695,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2718,33 +2730,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2753,33 +2765,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2788,33 +2800,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2823,33 +2835,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2858,33 +2870,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2893,33 +2905,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2928,33 +2940,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2963,33 +2975,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -2998,33 +3010,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3033,33 +3045,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3068,33 +3080,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3103,33 +3115,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3138,62 +3150,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3208,33 +3220,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3243,122 +3255,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>165</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>163</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3421,12 +3433,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3434,34 +3446,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3469,7 +3481,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3478,7 +3490,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3497,10 +3509,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3508,7 +3520,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3517,7 +3529,7 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3529,21 +3541,21 @@
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
-        <v>0.129032258064516</v>
+        <v>0.290322580645161</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3552,7 +3564,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3575,10 +3587,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3587,7 +3599,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3610,10 +3622,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3622,7 +3634,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3645,7 +3657,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3657,11 +3669,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.138211382113821</v>
+        <v>0.178861788617886</v>
       </c>
     </row>
   </sheetData>
@@ -3691,171 +3703,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3864,7 +3876,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3873,7 +3885,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3905,23 +3917,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,7 +3959,7 @@
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A6)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3960,7 +3972,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3973,7 +3985,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3986,7 +3998,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3999,7 +4011,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4012,7 +4024,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,7 +4037,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4038,7 +4050,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4051,7 +4063,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(match-service): catálogo de partidos con filtros combinables (HU-09)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="247">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -266,16 +266,22 @@
     <t xml:space="preserve">Como administrador, quiero registrar partidos (nombre, descripción, fecha, hora, estado, escenario) para publicarlos</t>
   </si>
   <si>
+    <t xml:space="preserve">Escenario inexistente → 404; fecha pasada rechazada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-08-partidos · PR #10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST/GET/PUT de partidos. Nace PROGRAMADO; fecha+hora pasadas (hora de Ecuador) → 422; estadio inexistente → 404. Máquina de estados en MatchStatus: PROGRAMADO→EN_CURSO→FINALIZADO y PROGRAMADO→CANCELADO; estados finales no se modifican (422). No se cambia de estadio (asientos reservados). No se eliminan partidos: se cancelan. Mass assignment de status bloqueado por DTO. 400 con mensaje claro para JSON/formato inválido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero consultar partidos filtrando por fecha, nombre o estadio para encontrar el evento que busco</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escenario inexistente → 404; fecha pasada rechazada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero consultar partidos filtrando por fecha, nombre o estadio para encontrar el evento que busco</t>
   </si>
   <si>
     <t xml:space="preserve">Consulta de partidos (2)</t>
@@ -1459,28 +1465,28 @@
                   <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>101</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1495,11 +1501,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="51158772"/>
-        <c:axId val="42992183"/>
+        <c:axId val="24728802"/>
+        <c:axId val="96046364"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="51158772"/>
+        <c:axId val="24728802"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1565,7 +1571,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42992183"/>
+        <c:crossAx val="96046364"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1573,7 +1579,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42992183"/>
+        <c:axId val="96046364"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1649,7 +1655,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51158772"/>
+        <c:crossAx val="24728802"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1977,7 +1983,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1986,7 +1992,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.178861788617886</v>
+        <v>0.203252032520325</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1995,7 +2001,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2395,7 +2401,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
         <v>77</v>
       </c>
@@ -2418,24 +2424,30 @@
         <v>59</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="I12" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>46314</v>
+      </c>
       <c r="J12" s="5" t="s">
         <v>68</v>
       </c>
       <c r="K12" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="L12" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
+      <c r="M12" s="15" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>66</v>
@@ -2453,30 +2465,30 @@
         <v>59</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2488,30 +2500,30 @@
         <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2523,30 +2535,30 @@
         <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2558,30 +2570,30 @@
         <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2593,30 +2605,30 @@
         <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2628,30 +2640,30 @@
         <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2660,33 +2672,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2695,33 +2707,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2730,33 +2742,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2765,33 +2777,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2800,33 +2812,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2835,33 +2847,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2870,33 +2882,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2905,33 +2917,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2940,33 +2952,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2975,33 +2987,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3010,33 +3022,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3045,33 +3057,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3080,33 +3092,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3115,33 +3127,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3150,62 +3162,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3220,33 +3232,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3255,122 +3267,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>167</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>165</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3433,12 +3445,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,34 +3458,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3481,7 +3493,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3490,7 +3502,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3509,10 +3521,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3520,7 +3532,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3529,7 +3541,7 @@
         <v>46314</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3541,21 +3553,21 @@
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
-        <v>0.290322580645161</v>
+        <v>0.387096774193548</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3564,7 +3576,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3587,10 +3599,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3599,7 +3611,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3622,10 +3634,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3634,7 +3646,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3657,7 +3669,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3669,11 +3681,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.178861788617886</v>
+        <v>0.203252032520325</v>
       </c>
     </row>
   </sheetData>
@@ -3703,171 +3715,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3876,7 +3888,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3885,7 +3897,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3917,23 +3929,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3972,7 +3984,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3985,7 +3997,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,7 +4010,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4011,7 +4023,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4024,7 +4036,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4037,7 +4049,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4050,7 +4062,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4063,7 +4075,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(auth-service): cambio de contraseña, roles en el JWT y administración de usuarios (HU-11, HU-12)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="256">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -281,45 +281,63 @@
     <t xml:space="preserve">Como cliente, quiero consultar partidos filtrando por fecha, nombre o estadio para encontrar el evento que busco</t>
   </si>
   <si>
+    <t xml:space="preserve">Consulta de partidos (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada filtro funciona solo y combinado; sin resultados → lista vacía, no error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-09-catalogo-partidos · PR #11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /matches con filtros opcionales y combinables (date, name, stadiumId, status) usando Specification. Sin filtros: PROGRAMADO desde hoy, orden por fecha y hora. Sin resultados → []. fetch del estadio contra N+1. Parámetros inválidos → 400 con lista errors. Pendiente: fijar idioma de mensajes (spring.web.locale: es).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero registrarme y recibir por correo mi username y contraseña de primer acceso para validar mi cuenta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS Usuarios/Auth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microservicio de autenticación (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correo inválido → 400; cédula/correo duplicado → 409; el correo llega con las credenciales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-14-swagger (rama compartida con HU-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auth-service creado (puerto 8081, auth_db). Registro: genera usuario (inicial + apellido, sin tildes, con número si existe) y contraseña temporal con SecureRandom; la envía por correo (Mailpit en desarrollo); nunca la devuelve en la API. Cédula ecuatoriana validada con módulo 10 (@CedulaEcuatoriana) y teléfono ecuatoriano. 409 por cédula o correo repetido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuario, quiero iniciar sesión y obtener un token según mi rol para acceder a mis funcionalidades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credenciales malas → 401 con mensaje genérico; usuario inactivo → 403; 5 intentos fallidos → BLOQUEADO 15 min (423); login exitoso reinicia el contador; token con rol y expiración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login con JWT HS256 (sub, role, userId, clientId, exp 60 min). 401 con mensaje genérico; 403 inactiva (se revisa después de la contraseña); 423 bloqueada; 5 intentos → BLOQUEADO 15 min con noRollbackFor; éxito reinicia el contador. Falta: cambio de contraseña de primer acceso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero gestionar usuarios y roles con estado ACTIVO/INACTIVO para controlar el acceso</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Consulta de partidos (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cada filtro funciona solo y combinado; sin resultados → lista vacía, no error</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero registrarme y recibir por correo mi username y contraseña de primer acceso para validar mi cuenta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS Usuarios/Auth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microservicio de autenticación (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correo inválido → 400; cédula/correo duplicado → 409; el correo llega con las credenciales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como usuario, quiero iniciar sesión y obtener un token según mi rol para acceder a mis funcionalidades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credenciales malas → 401 con mensaje genérico; usuario inactivo → 403; 5 intentos fallidos → BLOQUEADO 15 min (423); login exitoso reinicia el contador; token con rol y expiración</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero gestionar usuarios y roles con estado ACTIVO/INACTIVO para controlar el acceso</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cliente llamando endpoint admin → 403; usuario desactivado no puede iniciar sesión</t>
   </si>
   <si>
@@ -332,6 +350,9 @@
     <t xml:space="preserve">Ninguna contraseña en texto plano en BD; campos obligatorios vacíos → 400</t>
   </si>
   <si>
+    <t xml:space="preserve">Contraseñas solo como hash BCrypt ($2a$10$). DTOs validados con lista errors (400). Mensajes en español.</t>
+  </si>
+  <si>
     <t xml:space="preserve">HU-14</t>
   </si>
   <si>
@@ -345,6 +366,12 @@
   </si>
   <si>
     <t xml:space="preserve">/swagger-ui accesible en ambos servicios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-14-swagger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swagger en match-service con grupos Estadios, Secciones y Partidos (/swagger-ui.html). springdoc 3.x (Spring Boot 4). Falta: Swagger de auth-service y PR.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-15</t>
@@ -1044,7 +1071,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1088,6 +1115,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1465,28 +1500,28 @@
                   <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>98</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1501,11 +1536,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="24728802"/>
-        <c:axId val="96046364"/>
+        <c:axId val="20885108"/>
+        <c:axId val="55051324"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24728802"/>
+        <c:axId val="20885108"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1571,7 +1606,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96046364"/>
+        <c:crossAx val="55051324"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1579,7 +1614,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="96046364"/>
+        <c:axId val="55051324"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1655,7 +1690,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24728802"/>
+        <c:crossAx val="20885108"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1983,7 +2018,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1992,7 +2027,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.203252032520325</v>
+        <v>0.227642276422764</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2001,7 +2036,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2442,7 +2477,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
         <v>82</v>
       </c>
@@ -2465,30 +2500,36 @@
         <v>59</v>
       </c>
       <c r="H13" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>46314</v>
+      </c>
+      <c r="J13" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="5" t="s">
+      <c r="K13" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="L13" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-    </row>
-    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M13" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>33</v>
@@ -2500,30 +2541,34 @@
         <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-    </row>
-    <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>93</v>
+      </c>
+      <c r="L14" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="M14" s="15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>33</v>
@@ -2535,30 +2580,34 @@
         <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K15" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L15" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
+      <c r="M15" s="15" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>33</v>
@@ -2570,30 +2619,30 @@
         <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>33</v>
@@ -2605,30 +2654,34 @@
         <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-    </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>106</v>
+      </c>
+      <c r="L17" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="M17" s="15" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2640,30 +2693,34 @@
         <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I18" s="14"/>
       <c r="J18" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
+        <v>112</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="M18" s="15" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2672,33 +2729,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2707,33 +2764,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2742,33 +2799,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2777,33 +2834,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2812,33 +2869,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2847,33 +2904,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2882,33 +2939,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2917,33 +2974,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -2952,33 +3009,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -2987,33 +3044,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3022,33 +3079,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3057,33 +3114,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3092,33 +3149,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3127,33 +3184,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3162,62 +3219,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3232,33 +3289,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3267,122 +3324,122 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3390,13 +3447,13 @@
   </sheetData>
   <autoFilter ref="A4:M39"/>
   <conditionalFormatting sqref="H5:H39">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3445,12 +3502,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3458,34 +3515,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3493,7 +3550,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3502,7 +3559,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3521,10 +3578,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3532,16 +3589,16 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3553,21 +3610,21 @@
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
-        <v>0.387096774193548</v>
+        <v>0.483870967741936</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3576,7 +3633,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3599,10 +3656,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3611,7 +3668,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3634,10 +3691,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3646,7 +3703,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3669,7 +3726,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3681,11 +3738,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.203252032520325</v>
+        <v>0.227642276422764</v>
       </c>
     </row>
   </sheetData>
@@ -3715,171 +3772,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3888,7 +3945,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3897,7 +3954,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3929,23 +3986,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3984,7 +4041,7 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3997,7 +4054,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4010,7 +4067,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4023,7 +4080,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,7 +4093,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4049,7 +4106,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4062,7 +4119,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4075,7 +4132,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: cierre del Sprint 1 con resumen y plan actualizado
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="257">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -302,19 +302,16 @@
     <t xml:space="preserve">MS Usuarios/Auth</t>
   </si>
   <si>
-    <t xml:space="preserve">En curso</t>
-  </si>
-  <si>
     <t xml:space="preserve">Microservicio de autenticación (5)</t>
   </si>
   <si>
     <t xml:space="preserve">Correo inválido → 400; cédula/correo duplicado → 409; el correo llega con las credenciales</t>
   </si>
   <si>
-    <t xml:space="preserve">feature/HU-14-swagger (rama compartida con HU-14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auth-service creado (puerto 8081, auth_db). Registro: genera usuario (inicial + apellido, sin tildes, con número si existe) y contraseña temporal con SecureRandom; la envía por correo (Mailpit en desarrollo); nunca la devuelve en la API. Cédula ecuatoriana validada con módulo 10 (@CedulaEcuatoriana) y teléfono ecuatoriano. 409 por cédula o correo repetido.</t>
+    <t xml:space="preserve">feature/HU-14-swagger · PR de cierre del Sprint 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auth-service (8081, auth_db). Registro: usuario generado (inicial + apellido, sin tildes, con número si existe), contraseña temporal con SecureRandom enviada por correo (Mailpit), nunca devuelta por la API. @CedulaEcuatoriana (módulo 10) y teléfono ecuatoriano. 409 por cédula o correo repetido.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-11</t>
@@ -326,7 +323,7 @@
     <t xml:space="preserve">Credenciales malas → 401 con mensaje genérico; usuario inactivo → 403; 5 intentos fallidos → BLOQUEADO 15 min (423); login exitoso reinicia el contador; token con rol y expiración</t>
   </si>
   <si>
-    <t xml:space="preserve">Login con JWT HS256 (sub, role, userId, clientId, exp 60 min). 401 con mensaje genérico; 403 inactiva (se revisa después de la contraseña); 423 bloqueada; 5 intentos → BLOQUEADO 15 min con noRollbackFor; éxito reinicia el contador. Falta: cambio de contraseña de primer acceso.</t>
+    <t xml:space="preserve">Login JWT HS256 (sub, role, userId, clientId; 60 min). 401 genérico; 423 bloqueada (antes de la contraseña); 403 inactiva (después); 5 intentos → BLOQUEADO 15 min con noRollbackFor. Cambio de contraseña: usuario tomado del token. Bug encontrado vía Swagger: el endpoint de login no estaba expuesto.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-12</t>
@@ -335,55 +332,55 @@
     <t xml:space="preserve">Como administrador, quiero gestionar usuarios y roles con estado ACTIVO/INACTIVO para controlar el acceso</t>
   </si>
   <si>
+    <t xml:space="preserve">Cliente llamando endpoint admin → 403; usuario desactivado no puede iniciar sesión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo ADMIN: listar usuarios y roles, activar/desactivar. ACTIVO desbloquea. No se asigna BLOQUEADO a mano, no se desactiva la propia cuenta ni el rol ADMIN (422). Roles en el JWT → 401/403.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero contraseñas con hash BCrypt y DTOs validados para cumplir la seguridad pedida (CID/AAA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninguna contraseña en texto plano en BD; campos obligatorios vacíos → 400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contraseñas solo como hash BCrypt ($2a$10$). DTOs validados con lista errors (400), mensajes en español.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero Swagger/OpenAPI en Partidos y Auth para documentar las APIs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entregable Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/swagger-ui accesible en ambos servicios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swagger en match-service (8082) y auth-service (8081, con botón Authorize). Contrato docs/apis/auth-service.openapi.yaml para Apidog.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero ver la disponibilidad de asientos de un partido para elegir dónde sentarme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS Reservas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cliente llamando endpoint admin → 403; usuario desactivado no puede iniciar sesión</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero contraseñas con hash BCrypt y DTOs validados para cumplir la seguridad pedida (CID/AAA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ninguna contraseña en texto plano en BD; campos obligatorios vacíos → 400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contraseñas solo como hash BCrypt ($2a$10$). DTOs validados con lista errors (400). Mensajes en español.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero Swagger/OpenAPI en Partidos y Auth para documentar las APIs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entregable Backend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/swagger-ui accesible en ambos servicios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feature/HU-14-swagger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swagger en match-service con grupos Estadios, Secciones y Partidos (/swagger-ui.html). springdoc 3.x (Spring Boot 4). Falta: Swagger de auth-service y PR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero ver la disponibilidad de asientos de un partido para elegir dónde sentarme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS Reservas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
     <t xml:space="preserve">Realizar reserva (4)</t>
@@ -674,6 +671,14 @@
   </si>
   <si>
     <t xml:space="preserve">Partidos y Auth funcionando con Swagger, JWT y roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incremento: match-service (estadios, secciones con filas y asientos, partidos con máquina de estados, catálogo con filtros) y auth-service (registro con credenciales por correo, login JWT con bloqueo, administración de usuarios y roles), ambos con Swagger. 31/31 puntos. 8 bugs encontrados y corregidos con pruebas (valores límite, transición de estados, seguridad). Riesgo abierto: match-service aún no valida el JWT. Resumen completo en docs/sprints/sprint-1.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salió bien: se completaron las 10 historias y los dos microservicios funcionan.
+Costó: surgieron dudas con conceptos nuevos (Java, JPA, JWT) y con Git (rama equivocada).
+Acción de mejora: hacer las cosas más rápido: revisar la rama antes de empezar, cerrar cada HU con su PR y probar cada endpoint apenas esté listo.</t>
   </si>
   <si>
     <t xml:space="preserve">Microservicio Reservas</t>
@@ -1071,7 +1076,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1115,14 +1120,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1503,25 +1500,25 @@
                   <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>95</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1536,11 +1533,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="20885108"/>
-        <c:axId val="55051324"/>
+        <c:axId val="73551692"/>
+        <c:axId val="81805860"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="20885108"/>
+        <c:axId val="73551692"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1606,7 +1603,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55051324"/>
+        <c:crossAx val="81805860"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1614,7 +1611,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55051324"/>
+        <c:axId val="81805860"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1690,7 +1687,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20885108"/>
+        <c:crossAx val="73551692"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2018,7 +2015,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2027,7 +2024,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.227642276422764</v>
+        <v>0.357723577235772</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2036,7 +2033,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2518,7 +2515,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>88</v>
       </c>
@@ -2541,28 +2538,30 @@
         <v>59</v>
       </c>
       <c r="H14" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="J14" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I14" s="14"/>
-      <c r="J14" s="5" t="s">
+      <c r="K14" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="L14" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="L14" s="15" t="s">
+      <c r="M14" s="15" t="s">
         <v>94</v>
-      </c>
-      <c r="M14" s="15" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>66</v>
@@ -2580,28 +2579,30 @@
         <v>59</v>
       </c>
       <c r="H15" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="J15" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I15" s="14"/>
-      <c r="J15" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="K15" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="L15" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="M15" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="L15" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="M15" s="15" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="B16" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>66</v>
@@ -2619,24 +2620,30 @@
         <v>59</v>
       </c>
       <c r="H16" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L16" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="M16" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="I16" s="14"/>
-      <c r="J16" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>31</v>
@@ -2654,34 +2661,36 @@
         <v>59</v>
       </c>
       <c r="H17" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I17" s="14"/>
-      <c r="J17" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="K17" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L17" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="M17" s="15" t="s">
         <v>106</v>
-      </c>
-      <c r="L17" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="M17" s="15" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>33</v>
@@ -2693,34 +2702,36 @@
         <v>59</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="I18" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I18" s="14" t="n">
+        <v>46315</v>
+      </c>
       <c r="J18" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K18" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="K18" s="5" t="s">
+      <c r="L18" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="M18" s="15" t="s">
         <v>112</v>
-      </c>
-      <c r="L18" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="M18" s="15" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>33</v>
@@ -2729,33 +2740,33 @@
         <v>3</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K19" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>120</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>121</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>122</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>33</v>
@@ -2764,33 +2775,33 @@
         <v>8</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>126</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>33</v>
@@ -2799,33 +2810,33 @@
         <v>5</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>129</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>33</v>
@@ -2834,33 +2845,33 @@
         <v>5</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="K22" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>131</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>132</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>33</v>
@@ -2869,33 +2880,33 @@
         <v>3</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>33</v>
@@ -2904,33 +2915,33 @@
         <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K24" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="K24" s="5" t="s">
-        <v>138</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>33</v>
@@ -2939,33 +2950,33 @@
         <v>5</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2974,33 +2985,33 @@
         <v>3</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="K26" s="5" t="s">
         <v>145</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>146</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3009,33 +3020,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="K27" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>153</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>154</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3044,33 +3055,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>157</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3079,33 +3090,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="K29" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>161</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3114,33 +3125,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3149,33 +3160,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3184,33 +3195,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="K32" s="5" t="s">
         <v>168</v>
-      </c>
-      <c r="K32" s="5" t="s">
-        <v>169</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>171</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3219,62 +3230,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E34" s="11" t="s">
         <v>175</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>176</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="K34" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="K34" s="5" t="s">
-        <v>179</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>180</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>181</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3289,33 +3300,33 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>183</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>184</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>33</v>
@@ -3324,62 +3335,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="K36" s="5" t="s">
         <v>185</v>
-      </c>
-      <c r="K36" s="5" t="s">
-        <v>186</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>188</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>190</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>191</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3388,58 +3399,58 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3447,13 +3458,13 @@
   </sheetData>
   <autoFilter ref="A4:M39"/>
   <conditionalFormatting sqref="H5:H39">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3502,12 +3513,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3515,34 +3526,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3550,7 +3561,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3559,7 +3570,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3578,18 +3589,18 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="K5" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="K5" s="15" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3598,7 +3609,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3610,21 +3621,25 @@
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
-        <v>0.483870967741936</v>
-      </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
+        <v>1</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>214</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3633,7 +3648,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3656,10 +3671,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3668,7 +3683,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3691,10 +3706,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3703,7 +3718,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3726,7 +3741,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3738,11 +3753,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.227642276422764</v>
+        <v>0.357723577235772</v>
       </c>
     </row>
   </sheetData>
@@ -3772,171 +3787,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3945,7 +3960,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3954,7 +3969,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -3986,23 +4001,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4054,7 +4069,7 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,7 +4082,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4080,7 +4095,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4093,7 +4108,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4106,7 +4121,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4119,7 +4134,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4132,7 +4147,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gestion): avance del Sprint 2 (HU-15, HU-16, HU-22 en curso)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="262">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -380,33 +380,45 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realizar reserva (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asiento reservado aparece ocupado para ese partido y libre para otro partido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-22-reservation-service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidades Reservation/SeatLock/Ticket/Parameter. GET /matches/{id}/availability devuelve solo asientos ocupados (RESERVED, o HELD con reserva sin vencer) y refreshSeconds del parámetro. Sin @Transactional por la llamada remota. Smoke test 200 OK. Faltan: pruebas de vencimiento (35–37), partido sin reservas, 404, 401, 503.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero reservar hasta 6 asientos por partido para asistir con acompañantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microservicio de reservas (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.ª entrada → 422; asiento ocupado → 409; dos reservas simultáneas del mismo asiento → solo una gana; máximo leído de Parámetro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diseño entregado: POST /reservations y GET /reservations/{publicId}. Llamada a match-service fuera de la transacción (ReservationService) y escritura en ReservationWriter (@Transactional, por el proxy de Spring). Máximo por parámetro → 422, ocupado → 409 (consulta + UNIQUE con saveAndFlush), solo CLIENTE → 403, IDOR → 404. Código RES-AAAA-XXXXXX aleatorio. Contrato docs/apis/reservation-service.openapi.yaml (design-first). Faltan: implementar y 15 casos de prueba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como sistema, quiero liberar los asientos de reservas no confirmadas a tiempo para que vuelvan a estar disponibles</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Realizar reserva (4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asiento reservado aparece ocupado para ese partido y libre para otro partido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero reservar hasta 6 asientos por partido para asistir con acompañantes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microservicio de reservas (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.ª entrada → 422; asiento ocupado → 409; dos reservas simultáneas del mismo asiento → solo una gana; máximo leído de Parámetro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como sistema, quiero liberar los asientos de reservas no confirmadas a tiempo para que vuelvan a estar disponibles</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reserva pendiente pasado el tiempo del parámetro → EXPIRADA y asientos libres</t>
   </si>
   <si>
@@ -465,6 +477,9 @@
   </si>
   <si>
     <t xml:space="preserve">Asiento inexistente en Partidos → 404 desde Reservas; Partidos caído → error controlado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation-service (8083, reservation_db) valida el JWT de auth-service sin llamarlo (mismo secreto) y GET /me. match-service ahora exige JWT de ADMIN para escribir y expone POST /internal/seats/validate con X-Internal-Key (comparación MessageDigest.isEqual). Cliente RestClient con timeouts 2 s/3 s: 404 se propaga, caída → 503. Smoke test OK (servicio arriba). Faltan: pruebas 404/503 y PR.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-23</t>
@@ -1076,7 +1091,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1120,6 +1135,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1533,11 +1556,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="73551692"/>
-        <c:axId val="81805860"/>
+        <c:axId val="68782507"/>
+        <c:axId val="86819995"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="73551692"/>
+        <c:axId val="68782507"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1603,7 +1626,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81805860"/>
+        <c:crossAx val="86819995"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1611,7 +1634,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81805860"/>
+        <c:axId val="86819995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1687,7 +1710,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73551692"/>
+        <c:crossAx val="68782507"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2720,7 +2743,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
         <v>113</v>
       </c>
@@ -2752,15 +2775,19 @@
       <c r="K19" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="L19" s="15"/>
-      <c r="M19" s="15"/>
-    </row>
-    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L19" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
@@ -2782,20 +2809,24 @@
       </c>
       <c r="I20" s="14"/>
       <c r="J20" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
+        <v>125</v>
+      </c>
+      <c r="L20" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
@@ -2813,24 +2844,24 @@
         <v>116</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
@@ -2848,24 +2879,24 @@
         <v>116</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
@@ -2883,24 +2914,24 @@
         <v>116</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
         <v>118</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
@@ -2918,24 +2949,24 @@
         <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
@@ -2953,30 +2984,30 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
-    <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -2992,26 +3023,30 @@
       </c>
       <c r="I26" s="14"/>
       <c r="J26" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
+        <v>149</v>
+      </c>
+      <c r="L26" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="M26" s="15" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3020,33 +3055,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3055,33 +3090,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3090,33 +3125,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3125,33 +3160,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>118</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3160,33 +3195,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3195,33 +3230,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3230,62 +3265,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3300,27 +3335,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3335,62 +3370,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3399,7 +3434,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3408,24 +3443,24 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3434,23 +3469,23 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3458,13 +3493,13 @@
   </sheetData>
   <autoFilter ref="A4:M39"/>
   <conditionalFormatting sqref="H5:H39">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3513,12 +3548,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3526,34 +3561,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3561,7 +3596,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3570,7 +3605,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3589,10 +3624,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,7 +3635,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3609,7 +3644,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3628,10 +3663,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3639,7 +3674,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3648,7 +3683,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3671,10 +3706,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3683,7 +3718,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3706,10 +3741,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3718,7 +3753,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3741,7 +3776,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3787,171 +3822,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3960,7 +3995,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -3969,7 +4004,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4001,23 +4036,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs(gestion): HU-15, 16, 18 y 22 terminadas
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="262">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -380,19 +380,16 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">En curso</t>
-  </si>
-  <si>
     <t xml:space="preserve">Realizar reserva (4)</t>
   </si>
   <si>
     <t xml:space="preserve">Asiento reservado aparece ocupado para ese partido y libre para otro partido</t>
   </si>
   <si>
-    <t xml:space="preserve">feature/HU-22-reservation-service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entidades Reservation/SeatLock/Ticket/Parameter. GET /matches/{id}/availability devuelve solo asientos ocupados (RESERVED, o HELD con reserva sin vencer) y refreshSeconds del parámetro. Sin @Transactional por la llamada remota. Smoke test 200 OK. Faltan: pruebas de vencimiento (35–37), partido sin reservas, 404, 401, 503.</t>
+    <t xml:space="preserve">feature/HU-22-reservation-service · PR #14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidades Reservation/SeatLock/Ticket/Parameter. GET /matches/{id}/availability devuelve solo asientos ocupados (RESERVED, o HELD con reserva sin vencer) y refreshSeconds del parámetro. Sin @Transactional por la llamada remota. Probado: partido con y sin ocupados, vencimiento de la reserva semilla, 404, 401, 400, 503.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-16</t>
@@ -407,7 +404,7 @@
     <t xml:space="preserve">7.ª entrada → 422; asiento ocupado → 409; dos reservas simultáneas del mismo asiento → solo una gana; máximo leído de Parámetro</t>
   </si>
   <si>
-    <t xml:space="preserve">Diseño entregado: POST /reservations y GET /reservations/{publicId}. Llamada a match-service fuera de la transacción (ReservationService) y escritura en ReservationWriter (@Transactional, por el proxy de Spring). Máximo por parámetro → 422, ocupado → 409 (consulta + UNIQUE con saveAndFlush), solo CLIENTE → 403, IDOR → 404. Código RES-AAAA-XXXXXX aleatorio. Contrato docs/apis/reservation-service.openapi.yaml (design-first). Faltan: implementar y 15 casos de prueba.</t>
+    <t xml:space="preserve">POST /reservations y GET /reservations/{publicId}. Llamada a match-service fuera de la transacción (ReservationService) y escritura en ReservationWriter (@Transactional, por el proxy de Spring). Máximo por parámetro → 422 (valor límite 6 OK), ocupado → 409 (consulta + UNIQUE con saveAndFlush), partido no PROGRAMADO → 422, asiento de otro estadio → 404, solo CLIENTE → 403, reserva ajena → 404 (IDOR). Vencidas se liberan al reservar (flush antes del INSERT). Código RES-AAAA-XXXXXX aleatorio. Pendiente: prueba de concurrencia con k6 (Sprint 4).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-17</t>
@@ -434,6 +431,9 @@
     <t xml:space="preserve">1 ticket por asiento; código QR no secuencial ni repetido</t>
   </si>
   <si>
+    <t xml:space="preserve">POST /reservations/{publicId}/confirm: re-valida el partido en match-service, bloqueo pesimista (SELECT ... FOR UPDATE) contra doble clic, solo PENDIENTE y sin vencer (409), asientos HELD → RESERVED y 1 ticket ACTIVO por asiento. QR = 64 caracteres hex de SecureRandom, sin datos personales. GET /tickets/{publicId}/qr devuelve PNG (ZXing), ticket ajeno → 404.</t>
+  </si>
+  <si>
     <t xml:space="preserve">HU-19</t>
   </si>
   <si>
@@ -479,7 +479,7 @@
     <t xml:space="preserve">Asiento inexistente en Partidos → 404 desde Reservas; Partidos caído → error controlado</t>
   </si>
   <si>
-    <t xml:space="preserve">reservation-service (8083, reservation_db) valida el JWT de auth-service sin llamarlo (mismo secreto) y GET /me. match-service ahora exige JWT de ADMIN para escribir y expone POST /internal/seats/validate con X-Internal-Key (comparación MessageDigest.isEqual). Cliente RestClient con timeouts 2 s/3 s: 404 se propaga, caída → 503. Smoke test OK (servicio arriba). Faltan: pruebas 404/503 y PR.</t>
+    <t xml:space="preserve">reservation-service (8083, reservation_db) valida el JWT de auth-service sin llamarlo (mismo secreto) y GET /me. match-service exige JWT de ADMIN para escribir y expone POST /internal/seats/validate con X-Internal-Key (MessageDigest.isEqual). RestClient con timeouts 2 s/3 s: 404 se propaga, caída → 503 sin guardar nada y recuperación al volver. Bug de contrato: X-Internal-Key declarado como esquema de seguridad no llegaba como header en Apidog → parámetro de header.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-23</t>
@@ -1091,7 +1091,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1135,14 +1135,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1526,22 +1518,22 @@
                   <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>79</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1556,11 +1548,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="68782507"/>
-        <c:axId val="86819995"/>
+        <c:axId val="423124"/>
+        <c:axId val="97907435"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="68782507"/>
+        <c:axId val="423124"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1626,7 +1618,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86819995"/>
+        <c:crossAx val="97907435"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1634,7 +1626,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86819995"/>
+        <c:axId val="97907435"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1710,7 +1702,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68782507"/>
+        <c:crossAx val="423124"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2038,7 +2030,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>44</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2047,7 +2039,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.357723577235772</v>
+        <v>0.51219512195122</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,7 +2048,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2766,28 +2758,30 @@
         <v>116</v>
       </c>
       <c r="H19" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>46316</v>
+      </c>
+      <c r="J19" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="I19" s="14"/>
-      <c r="J19" s="5" t="s">
+      <c r="K19" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="L19" s="15" t="s">
+      <c r="M19" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="M19" s="15" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="B20" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>123</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>66</v>
@@ -2805,28 +2799,30 @@
         <v>116</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="I20" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>46316</v>
+      </c>
       <c r="J20" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="L20" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="M20" s="15" t="s">
         <v>125</v>
-      </c>
-      <c r="L20" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="M20" s="15" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>66</v>
@@ -2844,24 +2840,24 @@
         <v>116</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I21" s="14"/>
       <c r="J21" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
@@ -2879,17 +2875,23 @@
         <v>116</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="I22" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I22" s="14" t="n">
+        <v>46316</v>
+      </c>
       <c r="J22" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="K22" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="K22" s="5" t="s">
+      <c r="L22" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="M22" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
@@ -2914,11 +2916,11 @@
         <v>116</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>137</v>
@@ -2949,7 +2951,7 @@
         <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
@@ -2984,7 +2986,7 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
@@ -2996,7 +2998,7 @@
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
-    <row r="26" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
         <v>145</v>
       </c>
@@ -3019,9 +3021,11 @@
         <v>116</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="I26" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I26" s="14" t="n">
+        <v>46316</v>
+      </c>
       <c r="J26" s="5" t="s">
         <v>148</v>
       </c>
@@ -3029,7 +3033,7 @@
         <v>149</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
         <v>150</v>
@@ -3058,7 +3062,7 @@
         <v>154</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
@@ -3093,7 +3097,7 @@
         <v>154</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
@@ -3128,7 +3132,7 @@
         <v>154</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
@@ -3163,11 +3167,11 @@
         <v>154</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>166</v>
@@ -3198,11 +3202,11 @@
         <v>154</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>169</v>
@@ -3233,7 +3237,7 @@
         <v>154</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
@@ -3268,7 +3272,7 @@
         <v>154</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
@@ -3303,7 +3307,7 @@
         <v>181</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
@@ -3338,7 +3342,7 @@
         <v>181</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
@@ -3373,7 +3377,7 @@
         <v>181</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
@@ -3408,7 +3412,7 @@
         <v>181</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
@@ -3443,7 +3447,7 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
@@ -3478,11 +3482,11 @@
         <v>181</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
         <v>200</v>
@@ -3493,13 +3497,13 @@
   </sheetData>
   <autoFilter ref="A4:M39"/>
   <conditionalFormatting sqref="H5:H39">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3695,11 +3699,11 @@
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A7,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0</v>
+        <v>0.475</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
@@ -3788,11 +3792,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.357723577235772</v>
+        <v>0.51219512195122</v>
       </c>
     </row>
   </sheetData>
@@ -4117,7 +4121,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4130,7 +4134,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4143,7 +4147,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4156,7 +4160,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4169,7 +4173,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4182,7 +4186,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HU-17: expiración automática + fix de confirmar (HU-18)
## Qué incluye
- HU-17: tarea programada que vence reservas PENDIENTE de todos los partidos.
  Intervalo leído de EXPIRATION_JOB_SECONDS en cada ciclo (fail-safe a 60 s).
- Fix HU-18: LazyInitializationException al confirmar. La reserva quedaba
  CONFIRMADA pero el cliente recibía 500. Ahora la transacción devuelve DTOs.
- Refactor: Reservation.expire() centraliza la regla de expiración.
- Se elimina la copia del contrato en docs/sprints.

## Nota
ReservationWriter.java contiene cambios de HU-17 y del fix de HU-18
(mismo archivo, commit de HU-17).

## Pruebas
Expiración automática (log + BD), asientos liberados en disponibilidad,
confirmar reserva expirada → 409, confirmada no se toca, cambio de
intervalo sin reiniciar, parámetro inválido → 60 s. Regresión de crear
y confirmar OK.
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="264">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -386,7 +386,7 @@
     <t xml:space="preserve">Asiento reservado aparece ocupado para ese partido y libre para otro partido</t>
   </si>
   <si>
-    <t xml:space="preserve">feature/HU-22-reservation-service · PR #14</t>
+    <t xml:space="preserve">feature/HU-22-reservation-service · PR #14 y #15</t>
   </si>
   <si>
     <t xml:space="preserve">Entidades Reservation/SeatLock/Ticket/Parameter. GET /matches/{id}/availability devuelve solo asientos ocupados (RESERVED, o HELD con reserva sin vencer) y refreshSeconds del parámetro. Sin @Transactional por la llamada remota. Probado: partido con y sin ocupados, vencimiento de la reserva semilla, 404, 401, 400, 503.</t>
@@ -413,31 +413,37 @@
     <t xml:space="preserve">Como sistema, quiero liberar los asientos de reservas no confirmadas a tiempo para que vuelvan a estar disponibles</t>
   </si>
   <si>
+    <t xml:space="preserve">Reserva pendiente pasado el tiempo del parámetro → EXPIRADA y asientos libres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-17-expiracion-automatica · PR #16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarea programada (SchedulingConfigurer + Trigger propio): el intervalo se lee de EXPIRATION_JOB_SECONDS antes de cada ciclo, se cambia sin reiniciar; valor inválido o ausente → 60 s con warn (fail-safe). Vence las PENDIENTE de todos los partidos con SELECT ... FOR UPDATE (no choca con confirmar). Reservation.expire() centraliza la regla (modelo de dominio rico). Log solo cuando expira algo. Hallazgo SonarQube (java:S6809): auto-invocación de método @Transactional → expirePending privado. Mejora futura: ShedLock con varias instancias.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero un ticket electrónico con QR único por cada entrada para ingresar al estadio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código QR (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 ticket por asiento; código QR no secuencial ni repetido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST /reservations/{publicId}/confirm: re-valida el partido en match-service, bloqueo pesimista (SELECT ... FOR UPDATE) contra doble clic, solo PENDIENTE y sin vencer (409), asientos HELD → RESERVED y 1 ticket ACTIVO por asiento. QR = 64 caracteres hex de SecureRandom, sin datos personales. GET /tickets/{publicId}/qr devuelve PNG (ZXing), ticket ajeno → 404. Bug encontrado en regresión (corregido en PR #16): LazyInitializationException al armar la respuesta fuera de la transacción → la reserva quedaba CONFIRMADA pero el cliente recibía 500. Regla: la transacción devuelve DTOs, no entidades.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente o administrador, quiero cancelar reservas activas no expiradas ni utilizadas para liberar asientos</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva pendiente pasado el tiempo del parámetro → EXPIRADA y asientos libres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero un ticket electrónico con QR único por cada entrada para ingresar al estadio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código QR (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 ticket por asiento; código QR no secuencial ni repetido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POST /reservations/{publicId}/confirm: re-valida el partido en match-service, bloqueo pesimista (SELECT ... FOR UPDATE) contra doble clic, solo PENDIENTE y sin vencer (409), asientos HELD → RESERVED y 1 ticket ACTIVO por asiento. QR = 64 caracteres hex de SecureRandom, sin datos personales. GET /tickets/{publicId}/qr devuelve PNG (ZXing), ticket ajeno → 404.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente o administrador, quiero cancelar reservas activas no expiradas ni utilizadas para liberar asientos</t>
   </si>
   <si>
     <t xml:space="preserve">Cancelar reserva EXPIRADA o UTILIZADA → 409; cliente no cancela reservas ajenas → 403</t>
@@ -1518,22 +1524,22 @@
                   <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>60</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1548,11 +1554,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="423124"/>
-        <c:axId val="97907435"/>
+        <c:axId val="91351235"/>
+        <c:axId val="27003731"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="423124"/>
+        <c:axId val="91351235"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1618,7 +1624,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97907435"/>
+        <c:crossAx val="27003731"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1626,7 +1632,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97907435"/>
+        <c:axId val="27003731"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1702,7 +1708,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="423124"/>
+        <c:crossAx val="91351235"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2030,7 +2036,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2039,7 +2045,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.51219512195122</v>
+        <v>0.552845528455285</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2048,7 +2054,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2817,7 +2823,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
         <v>126</v>
       </c>
@@ -2840,24 +2846,30 @@
         <v>116</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="I21" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I21" s="14" t="n">
+        <v>46316</v>
+      </c>
       <c r="J21" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K21" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="L21" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
-    </row>
-    <row r="22" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M21" s="15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>66</v>
@@ -2881,24 +2893,24 @@
         <v>46316</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L22" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>66</v>
@@ -2916,24 +2928,24 @@
         <v>116</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I23" s="14"/>
       <c r="J23" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
@@ -2951,24 +2963,24 @@
         <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
@@ -2986,30 +2998,30 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -3027,30 +3039,30 @@
         <v>46316</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3059,33 +3071,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3094,33 +3106,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3129,33 +3141,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3164,33 +3176,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3199,33 +3211,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3234,33 +3246,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3269,62 +3281,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3339,27 +3351,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3374,62 +3386,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>182</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>180</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3438,7 +3450,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3447,24 +3459,24 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3473,23 +3485,23 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3552,12 +3564,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3565,34 +3577,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,7 +3612,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3609,7 +3621,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3628,10 +3640,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3639,7 +3651,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3648,7 +3660,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3667,10 +3679,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3678,7 +3690,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3687,7 +3699,7 @@
         <v>46316</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3699,21 +3711,21 @@
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A7,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0.475</v>
+        <v>0.6</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46317</v>
@@ -3722,7 +3734,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3745,10 +3757,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3757,7 +3769,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3780,7 +3792,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3792,11 +3804,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.51219512195122</v>
+        <v>0.552845528455285</v>
       </c>
     </row>
   </sheetData>
@@ -3826,171 +3838,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -3999,7 +4011,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4008,7 +4020,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4040,23 +4052,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4121,7 +4133,7 @@
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4134,7 +4146,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4147,7 +4159,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4160,7 +4172,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4173,7 +4185,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4186,7 +4198,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: contrato de cancelación y replanificación del Sprint 2 (HU-19)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="266">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -446,7 +446,10 @@
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Cancelar reserva EXPIRADA o UTILIZADA → 409; cliente no cancela reservas ajenas → 403</t>
+    <t xml:space="preserve">Cancelar reserva EXPIRADA o UTILIZADA → 409; reserva ajena → 404 (no revela que existe, igual que consultar y confirmar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisión 21-oct: reserva ajena → 404 y no 403, por consistencia con GET y confirmar (anti-IDOR / anti-enumeración). Criterio de aceptación actualizado.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-20</t>
@@ -624,6 +627,9 @@
   </si>
   <si>
     <t xml:space="preserve">Login, cancelación y cambios de estado quedan registrados con usuario, acción y fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should. Recortable: si no alcanza el tiempo, se documenta como trabajo futuro (decisión de alcance del Sprint 2, replanificado el 21-oct).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-35</t>
@@ -1554,11 +1560,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="91351235"/>
-        <c:axId val="27003731"/>
+        <c:axId val="61798583"/>
+        <c:axId val="70509305"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="91351235"/>
+        <c:axId val="61798583"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1624,7 +1630,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27003731"/>
+        <c:crossAx val="70509305"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1632,7 +1638,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27003731"/>
+        <c:axId val="70509305"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1708,7 +1714,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91351235"/>
+        <c:crossAx val="61798583"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2905,7 +2911,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>136</v>
       </c>
@@ -2938,14 +2944,16 @@
         <v>139</v>
       </c>
       <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
+      <c r="M23" s="15" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>66</v>
@@ -2967,20 +2975,20 @@
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
@@ -3002,26 +3010,26 @@
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -3039,30 +3047,30 @@
         <v>46316</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3071,33 +3079,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H27" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3106,7 +3114,7 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H28" s="13" t="s">
         <v>138</v>
@@ -3116,23 +3124,23 @@
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3141,33 +3149,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H29" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3176,7 +3184,7 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H30" s="13" t="s">
         <v>138</v>
@@ -3186,23 +3194,23 @@
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3211,7 +3219,7 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H31" s="13" t="s">
         <v>138</v>
@@ -3221,23 +3229,23 @@
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3246,33 +3254,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3281,62 +3289,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H34" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3351,7 +3359,7 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H35" s="13" t="s">
         <v>138</v>
@@ -3361,17 +3369,17 @@
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3386,62 +3394,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H36" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H37" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3450,7 +3458,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3466,17 +3474,19 @@
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
+      <c r="M38" s="15" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3485,13 +3495,13 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H39" s="13" t="s">
         <v>138</v>
@@ -3501,7 +3511,7 @@
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
@@ -3564,12 +3574,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3577,34 +3587,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3612,7 +3622,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3621,7 +3631,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
@@ -3640,10 +3650,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3651,7 +3661,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3660,7 +3670,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
@@ -3679,10 +3689,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3690,16 +3700,16 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
@@ -3722,19 +3732,19 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="C8" s="4" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
@@ -3757,10 +3767,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3769,7 +3779,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
@@ -3792,7 +3802,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3838,171 +3848,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4011,7 +4021,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4020,7 +4030,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4052,23 +4062,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs: actualización de sprint y servicio refactor(app):  cambio de nivel de properties
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Burndown" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$39</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="275">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -443,21 +443,24 @@
     <t xml:space="preserve">Como cliente o administrador, quiero cancelar reservas activas no expiradas ni utilizadas para liberar asientos</t>
   </si>
   <si>
+    <t xml:space="preserve">Cancelar reserva EXPIRADA o UTILIZADA → 409; reserva ajena → 404 (no revela que existe, igual que consultar y confirmar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-19-cancelar-reserva · PR #17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST /reservations/{publicId}/cancel (borrado lógico: la reserva queda CANCELADA para reportes y auditoría). Dueño o ADMIN; ajena → 404 (decisión 21-oct, consistente con consultar y confirmar). Cancelada/expirada/vencida o con entrada UTILIZADO → 409. CONFIRMADA de partido EN_CURSO/FINALIZADO → 422; PENDIENTE se cancela aunque match-service esté caído (sin dependencia innecesaria). Reservation.cancel() libera asientos y anula tickets; mismo bloqueo pesimista que confirmar y expirar. Refactor findAccessible (regla anti-IDOR en un solo lugar) y MeController movido a controller. Integración probada: al cancelar se libera el cupo de 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero un reporte "Mis reservas" con historial, tickets y estado, descargable en PDF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Cancelar reserva EXPIRADA o UTILIZADA → 409; reserva ajena → 404 (no revela que existe, igual que consultar y confirmar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decisión 21-oct: reserva ajena → 404 y no 403, por consistencia con GET y confirmar (anti-IDOR / anti-enumeración). Criterio de aceptación actualizado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero un reporte "Mis reservas" con historial, tickets y estado, descargable en PDF</t>
-  </si>
-  <si>
     <t xml:space="preserve">Implementación aplicación web (10)</t>
   </si>
   <si>
@@ -642,6 +645,30 @@
   </si>
   <si>
     <t xml:space="preserve">Dos POST con la misma Idempotency-Key devuelven la misma reserva, sin duplicar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero cancelar solo algunas entradas de una reserva confirmada para no perder los asientos de mis acompañantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anular 1 ticket → ANULADO y asiento libre; la reserva sigue CONFIRMADA con las demás; al anular la última pasa a CANCELADA; el cupo de 6 se libera; ticket UTILIZADO → 409; ticket ajeno → 404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hueco funcional encontrado al probar HU-19 (21-oct): el requisito habla de cancelar reservas, no entradas. Decisión: HU-19 cancela la reserva completa; la cancelación parcial queda como Could. Alternativa mientras tanto: hacer reservas separadas por grupo. El diseño ya lo soporta (el conteo de 6 usa seat_lock). Documentar en README → Supuestos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero descargar mis entradas en PDF, una por página con su código QR, para presentarlas en la puerta sin depender de internet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una página por ticket ACTIVO con partido, estadio, fecha, asiento, código de reserva y QR legible por el celular; reserva sin entradas activas → 409; reserva ajena → 404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedido de la usuaria al probar HU-20 (22-oct): ver el QR de cada asiento también en PDF, tipo pase de abordar. Endpoint aparte del historial (GET /reservations/{publicId}/tickets/pdf) para no inflar el PDF de Mis reservas con imágenes. Reutiliza QrCodeGenerator y la búsqueda de partido con degradación elegante.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprints</t>
@@ -1386,31 +1413,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>123</c:v>
+                  <c:v>129</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>109.333333333333</c:v>
+                  <c:v>114.666666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>95.6666666666667</c:v>
+                  <c:v>100.333333333333</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>82</c:v>
+                  <c:v>86</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>68.3333333333333</c:v>
+                  <c:v>71.6666666666667</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>54.6666666666667</c:v>
+                  <c:v>57.3333333333333</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>41</c:v>
+                  <c:v>43</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>27.3333333333333</c:v>
+                  <c:v>28.6666666666667</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13.6666666666667</c:v>
+                  <c:v>14.3333333333333</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1518,34 +1545,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>110</c:v>
+                  <c:v>116</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>101</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>95</c:v>
-                </c:pt>
                 <c:pt idx="3">
-                  <c:v>79</c:v>
+                  <c:v>85</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>55</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1560,11 +1587,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="61798583"/>
-        <c:axId val="70509305"/>
+        <c:axId val="18013576"/>
+        <c:axId val="41127647"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="61798583"/>
+        <c:axId val="18013576"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1630,7 +1657,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70509305"/>
+        <c:crossAx val="41127647"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1638,7 +1665,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="70509305"/>
+        <c:axId val="41127647"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1714,7 +1741,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61798583"/>
+        <c:crossAx val="18013576"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2023,8 +2050,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTA('Product Backlog'!A5:A39)</f>
-        <v>35</v>
+        <f aca="false">COUNTA('Product Backlog'!A5:A41)</f>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2032,8 +2059,8 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">SUM('Product Backlog'!F5:F39)</f>
-        <v>123</v>
+        <f aca="false">SUM('Product Backlog'!F5:F41)</f>
+        <v>129</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2041,8 +2068,8 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!F5:F39,'Product Backlog'!H5:H39,"Hecho")</f>
-        <v>68</v>
+        <f aca="false">SUMIFS('Product Backlog'!F5:F41,'Product Backlog'!H5:H41,"Hecho")</f>
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2051,7 +2078,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.552845528455285</v>
+        <v>0.550387596899225</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2059,8 +2086,8 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!H5:H39,"Hecho")</f>
-        <v>19</v>
+        <f aca="false">COUNTIF('Product Backlog'!H5:H41,"Hecho")</f>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2104,7 +2131,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -2911,7 +2938,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>136</v>
       </c>
@@ -2934,16 +2961,20 @@
         <v>116</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="I23" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I23" s="14" t="n">
+        <v>46316</v>
+      </c>
       <c r="J23" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K23" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="L23" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="L23" s="15"/>
       <c r="M23" s="15" t="s">
         <v>140</v>
       </c>
@@ -2971,24 +3002,24 @@
         <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
@@ -3006,30 +3037,30 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -3047,30 +3078,30 @@
         <v>46316</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3079,33 +3110,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3114,33 +3145,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3149,33 +3180,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3184,33 +3215,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3219,33 +3250,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3254,33 +3285,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3289,62 +3320,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3359,27 +3390,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3394,62 +3425,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3458,7 +3489,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3467,26 +3498,26 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3495,30 +3526,104 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
+    <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="F40" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="H40" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="I40" s="14"/>
+      <c r="J40" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K40" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F41" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="H41" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="I41" s="14"/>
+      <c r="J41" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="K41" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="L41" s="15"/>
+      <c r="M41" s="15" t="s">
+        <v>213</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M39"/>
-  <conditionalFormatting sqref="H5:H39">
+  <autoFilter ref="A4:M41"/>
+  <conditionalFormatting sqref="H5:H41">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Hecho"</formula>
     </cfRule>
@@ -3530,15 +3635,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H39" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H41" type="list">
       <formula1>"Pendiente,En curso,Hecho,Bloqueado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G39" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G41" type="list">
       <formula1>Sprints!$A$5:$A$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I39" type="date">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I41" type="date">
       <formula1>DATE(2026,10,17)</formula1>
       <formula2>DATE(2026,10,26)</formula2>
     </dataValidation>
@@ -3574,12 +3679,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,34 +3692,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3622,7 +3727,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3631,18 +3736,18 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A5)</f>
         <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A5)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A5)</f>
         <v>13</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A5,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A5,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
@@ -3650,10 +3755,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3661,7 +3766,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3670,18 +3775,18 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A6)</f>
         <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A6)</f>
         <v>31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A6,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A6,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
         <v>31</v>
       </c>
       <c r="I6" s="6" t="n">
@@ -3689,10 +3794,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3700,7 +3805,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3709,33 +3814,33 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A7)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A7)</f>
+        <v>10</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A7)</f>
-        <v>40</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A7)</f>
+        <v>43</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A7,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
-        <v>24</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A7,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
+        <v>27</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0.6</v>
+        <v>0.627906976744186</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>157</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46318</v>
@@ -3744,18 +3849,18 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="F8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A8)</f>
         <v>7</v>
       </c>
       <c r="G8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A8)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A8)</f>
         <v>26</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A8,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A8,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
         <v>0</v>
       </c>
       <c r="I8" s="6" t="n">
@@ -3767,10 +3872,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3779,18 +3884,18 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="F9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$39,A9)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A9)</f>
+        <v>6</v>
       </c>
       <c r="G9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A9)</f>
-        <v>13</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A9)</f>
+        <v>16</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$G$5:$G$39,A9,'Product Backlog'!$H$5:$H$39,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A9,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
         <v>0</v>
       </c>
       <c r="I9" s="6" t="n">
@@ -3802,23 +3907,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G10" s="3" t="n">
         <f aca="false">SUM(G5:G9)</f>
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.552845528455285</v>
+        <v>0.550387596899225</v>
       </c>
     </row>
   </sheetData>
@@ -3848,171 +3953,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4021,7 +4126,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4030,7 +4135,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4062,23 +4167,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4087,11 +4192,11 @@
       </c>
       <c r="B5" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-0/9)</f>
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A5)</f>
-        <v>110</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A5)</f>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4100,11 +4205,11 @@
       </c>
       <c r="B6" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-1/9)</f>
-        <v>109.333333333333</v>
+        <v>114.666666666667</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A6)</f>
-        <v>101</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A6)</f>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4113,11 +4218,11 @@
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-2/9)</f>
-        <v>95.6666666666667</v>
+        <v>100.333333333333</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A7)</f>
-        <v>95</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A7)</f>
+        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4126,11 +4231,11 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-3/9)</f>
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A8)</f>
-        <v>79</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A8)</f>
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,11 +4244,11 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-4/9)</f>
-        <v>68.3333333333333</v>
+        <v>71.6666666666667</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A9)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A9)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4152,11 +4257,11 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-5/9)</f>
-        <v>54.6666666666667</v>
+        <v>57.3333333333333</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A10)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A10)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4165,11 +4270,11 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-6/9)</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A11)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A11)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4178,11 +4283,11 @@
       </c>
       <c r="B12" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-7/9)</f>
-        <v>27.3333333333333</v>
+        <v>28.6666666666667</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A12)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A12)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4191,11 +4296,11 @@
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-8/9)</f>
-        <v>13.6666666666667</v>
+        <v>14.3333333333333</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A13)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A13)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4207,8 +4312,8 @@
         <v>0</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$39,'Product Backlog'!$H$5:$H$39,"Hecho",'Product Backlog'!$I$5:$I$39,"&lt;="&amp;A14)</f>
-        <v>55</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A14)</f>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: contrato de entradas en PDF y HU-20 terminada
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="277">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -458,19 +458,25 @@
     <t xml:space="preserve">Como cliente, quiero un reporte "Mis reservas" con historial, tickets y estado, descargable en PDF</t>
   </si>
   <si>
+    <t xml:space="preserve">Implementación aplicación web (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo muestra reservas propias; PDF se genera y abre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-20-mis-reservas-pdf · PR #18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /reservations/me (JSON) y /me/pdf (OpenPDF): historial del cliente del token (seguridad por diseño: no recibe id), de la más nueva a la más antigua. Datos del partido pedidos a match-service una vez por partido distinto, fuera de la transacción; si no responde → match null / "información no disponible" (degradación elegante). N+1 local resuelto con default_batch_fetch_size (bug de configuración: estaba bajo spring.jpa.hibernate y se ignoraba sin error). ADMIN → 403. Limitación del modelo: reservas canceladas/expiradas sin confirmar no conservan sus asientos (seat_lock es el candado vigente, no historial). Hallazgos Sonar: throws Exception sobrante, CSRF documentado (S4502), literales de rol (S1192).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero un reporte consolidado con filtros (fechas, partido, estado) e indicadores de ocupación, en PDF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementación aplicación web (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo muestra reservas propias; PDF se genera y abre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero un reporte consolidado con filtros (fechas, partido, estado) e indicadores de ocupación, en PDF</t>
   </si>
   <si>
     <t xml:space="preserve">Ocupación por partido y por sección calculada correctamente; filtros combinables</t>
@@ -1560,19 +1566,19 @@
                   <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1587,11 +1593,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="18013576"/>
-        <c:axId val="41127647"/>
+        <c:axId val="42629394"/>
+        <c:axId val="6333586"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="18013576"/>
+        <c:axId val="42629394"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1657,7 +1663,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41127647"/>
+        <c:crossAx val="6333586"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1665,7 +1671,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41127647"/>
+        <c:axId val="6333586"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1741,7 +1747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18013576"/>
+        <c:crossAx val="42629394"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2069,7 +2075,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F41,'Product Backlog'!H5:H41,"Hecho")</f>
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2078,7 +2084,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.550387596899225</v>
+        <v>0.589147286821706</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2087,7 +2093,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H41,"Hecho")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2979,7 +2985,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="204.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
         <v>141</v>
       </c>
@@ -3002,24 +3008,30 @@
         <v>116</v>
       </c>
       <c r="H24" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>46317</v>
+      </c>
+      <c r="J24" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="I24" s="14"/>
-      <c r="J24" s="5" t="s">
+      <c r="K24" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="K24" s="5" t="s">
+      <c r="L24" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
+      <c r="M24" s="15" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>66</v>
@@ -3037,30 +3049,30 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I25" s="14"/>
       <c r="J25" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -3078,30 +3090,30 @@
         <v>46316</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3110,33 +3122,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3145,33 +3157,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3180,33 +3192,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3215,33 +3227,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3250,33 +3262,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3285,33 +3297,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3320,62 +3332,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3390,27 +3402,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3425,62 +3437,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>186</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>184</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3489,7 +3501,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3498,26 +3510,26 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I38" s="14"/>
       <c r="J38" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3526,33 +3538,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3561,35 +3573,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3598,7 +3610,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3607,18 +3619,18 @@
         <v>116</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I41" s="14"/>
       <c r="J41" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="L41" s="15"/>
       <c r="M41" s="15" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -3679,12 +3691,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3692,34 +3704,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,7 +3739,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3736,7 +3748,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A5)</f>
@@ -3755,10 +3767,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3766,7 +3778,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3775,7 +3787,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A6)</f>
@@ -3794,10 +3806,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3805,7 +3817,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3814,7 +3826,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A7)</f>
@@ -3826,21 +3838,21 @@
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A7,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0.627906976744186</v>
+        <v>0.744186046511628</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46318</v>
@@ -3849,7 +3861,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A8)</f>
@@ -3872,10 +3884,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3884,7 +3896,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A9)</f>
@@ -3907,7 +3919,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3919,11 +3931,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.550387596899225</v>
+        <v>0.589147286821706</v>
       </c>
     </row>
   </sheetData>
@@ -3953,171 +3965,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4126,7 +4138,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4135,7 +4147,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4167,23 +4179,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4261,7 +4273,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A10)</f>
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4274,7 +4286,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A11)</f>
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4287,7 +4299,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A12)</f>
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4300,7 +4312,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A13)</f>
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4313,7 +4325,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A14)</f>
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(reservation-service): contrato del reporte del administrador (HU-21)
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Burndown" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$41</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$43</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="286">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -674,7 +674,34 @@
     <t xml:space="preserve">Una página por ticket ACTIVO con partido, estadio, fecha, asiento, código de reserva y QR legible por el celular; reserva sin entradas activas → 409; reserva ajena → 404</t>
   </si>
   <si>
-    <t xml:space="preserve">Pedido de la usuaria al probar HU-20 (22-oct): ver el QR de cada asiento también en PDF, tipo pase de abordar. Endpoint aparte del historial (GET /reservations/{publicId}/tickets/pdf) para no inflar el PDF de Mis reservas con imágenes. Reutiliza QrCodeGenerator y la búsqueda de partido con degradación elegante.</t>
+    <t xml:space="preserve">feature/HU-37-entradas-pdf · PR #19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /reservations/{publicId}/tickets/pdf: una página A6 por ticket ACTIVO con partido, estadio, fecha, asiento, código de reserva y QR (mismo QrCodeGenerator que /tickets/{id}/qr). Escaneado con el celular: coincide con qrCode. Reserva ajena → 404 (reutiliza findOne), sin entradas activas → 409 en JSON (tipo PDF solo en la respuesta exitosa, no con produces). Refactor: MatchLookup reutilizable (historial y entradas). Hallazgo de pruebas: variable genérica public_id en Apidog mezclaba id de reserva y de ticket → variables reservationId y ticketId.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero ubicar cada sección como un recuadro sobre el plano del estadio para que el cliente vea un mapa real y elija su asiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sección guarda x, y, ancho y alto en % del plano (0–100); fuera del plano → 400; superpuesta con otra sección → 422; GET /stadiums/{id}/layout devuelve secciones con su recuadro, filas y asientos; semillas con coordenadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea de la usuaria (22-oct): al crear secciones, ubicarlas como recuadros sobre el plano, porque un enum de lado (norte/sur/...) no representa estadios reales. Geometría en porcentaje para que el mapa escale a cualquier pantalla. Incluye el endpoint /layout pendiente desde HU-07. Requisito del mapa de asientos del frontend. Primero: formulario con vista previa en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero arrastrar y redimensionar las secciones sobre el plano en lugar de escribir coordenadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrastrar/redimensionar actualiza x, y, ancho y alto; se guarda con el mismo endpoint de HU-38; las reglas de superposición siguen validándose en el backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejora visual de HU-38: editor de arrastrar y soltar (por ejemplo react-rnd). Recortable: HU-38 ya permite ubicar las secciones con números y vista previa.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprints</t>
@@ -1419,31 +1446,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>129</c:v>
+                  <c:v>137</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>114.666666666667</c:v>
+                  <c:v>121.777777777778</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100.333333333333</c:v>
+                  <c:v>106.555555555556</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>86</c:v>
+                  <c:v>91.3333333333333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>71.6666666666667</c:v>
+                  <c:v>76.1111111111111</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>57.3333333333333</c:v>
+                  <c:v>60.8888888888889</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>43</c:v>
+                  <c:v>45.6666666666667</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>28.6666666666667</c:v>
+                  <c:v>30.4444444444444</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>14.3333333333333</c:v>
+                  <c:v>15.2222222222222</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1551,34 +1578,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>116</c:v>
+                  <c:v>124</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>107</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>101</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>85</c:v>
+                  <c:v>93</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>58</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>53</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>53</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>53</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>53</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>53</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1593,11 +1620,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="42629394"/>
-        <c:axId val="6333586"/>
+        <c:axId val="87482277"/>
+        <c:axId val="88605805"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="42629394"/>
+        <c:axId val="87482277"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1663,7 +1690,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6333586"/>
+        <c:crossAx val="88605805"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1671,7 +1698,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6333586"/>
+        <c:axId val="88605805"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1747,7 +1774,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42629394"/>
+        <c:crossAx val="87482277"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2056,8 +2083,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTA('Product Backlog'!A5:A41)</f>
-        <v>37</v>
+        <f aca="false">COUNTA('Product Backlog'!A5:A43)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2065,8 +2092,8 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">SUM('Product Backlog'!F5:F41)</f>
-        <v>129</v>
+        <f aca="false">SUM('Product Backlog'!F5:F43)</f>
+        <v>137</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2074,8 +2101,8 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!F5:F41,'Product Backlog'!H5:H41,"Hecho")</f>
-        <v>76</v>
+        <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2084,7 +2111,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.589147286821706</v>
+        <v>0.576642335766423</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2092,8 +2119,8 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!H5:H41,"Hecho")</f>
-        <v>21</v>
+        <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
+        <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2137,7 +2164,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3596,7 +3623,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
         <v>212</v>
       </c>
@@ -3619,23 +3646,101 @@
         <v>116</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="I41" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I41" s="14" t="n">
+        <v>46317</v>
+      </c>
       <c r="J41" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="L41" s="15"/>
+      <c r="L41" s="15" t="s">
+        <v>215</v>
+      </c>
       <c r="M41" s="15" t="s">
-        <v>215</v>
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="H42" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="I42" s="14"/>
+      <c r="J42" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K42" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="L42" s="15"/>
+      <c r="M42" s="15" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="F43" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="H43" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="I43" s="14"/>
+      <c r="J43" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="L43" s="15"/>
+      <c r="M43" s="15" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M41"/>
-  <conditionalFormatting sqref="H5:H41">
+  <autoFilter ref="A4:M43"/>
+  <conditionalFormatting sqref="H5:H43">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Hecho"</formula>
     </cfRule>
@@ -3647,15 +3752,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H41" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H43" type="list">
       <formula1>"Pendiente,En curso,Hecho,Bloqueado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G41" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
       <formula1>Sprints!$A$5:$A$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I41" type="date">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I43" type="date">
       <formula1>DATE(2026,10,17)</formula1>
       <formula2>DATE(2026,10,26)</formula2>
     </dataValidation>
@@ -3691,12 +3796,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3704,34 +3809,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3739,7 +3844,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3748,18 +3853,18 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
         <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A5)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A5)</f>
         <v>13</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A5,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A5,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
@@ -3767,10 +3872,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3778,7 +3883,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3787,18 +3892,18 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
         <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A6)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A6)</f>
         <v>31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A6,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A6,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
         <v>31</v>
       </c>
       <c r="I6" s="6" t="n">
@@ -3806,10 +3911,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3817,7 +3922,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3826,23 +3931,23 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
         <v>10</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A7)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A7)</f>
         <v>43</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A7,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
-        <v>32</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A7,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
+        <v>35</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0.744186046511628</v>
+        <v>0.813953488372093</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
@@ -3861,18 +3966,18 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="F8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A8)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
+        <v>8</v>
       </c>
       <c r="G8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A8)</f>
-        <v>26</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8)</f>
+        <v>31</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A8,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
         <v>0</v>
       </c>
       <c r="I8" s="6" t="n">
@@ -3887,7 +3992,7 @@
         <v>187</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -3896,18 +4001,18 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$41,A9)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
+        <v>7</v>
       </c>
       <c r="G9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A9)</f>
-        <v>16</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A9)</f>
+        <v>19</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$G$5:$G$41,A9,'Product Backlog'!$H$5:$H$41,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A9,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
         <v>0</v>
       </c>
       <c r="I9" s="6" t="n">
@@ -3919,23 +4024,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G10" s="3" t="n">
         <f aca="false">SUM(G5:G9)</f>
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.589147286821706</v>
+        <v>0.576642335766423</v>
       </c>
     </row>
   </sheetData>
@@ -3965,104 +4070,104 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
@@ -4073,63 +4178,63 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4138,7 +4243,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4147,7 +4252,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4179,23 +4284,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4204,11 +4309,11 @@
       </c>
       <c r="B5" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-0/9)</f>
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A5)</f>
-        <v>116</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A5)</f>
+        <v>124</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4217,11 +4322,11 @@
       </c>
       <c r="B6" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-1/9)</f>
-        <v>114.666666666667</v>
+        <v>121.777777777778</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A6)</f>
-        <v>107</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A6)</f>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4230,11 +4335,11 @@
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-2/9)</f>
-        <v>100.333333333333</v>
+        <v>106.555555555556</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A7)</f>
-        <v>101</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A7)</f>
+        <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4243,11 +4348,11 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-3/9)</f>
-        <v>86</v>
+        <v>91.3333333333333</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A8)</f>
-        <v>85</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A8)</f>
+        <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4256,11 +4361,11 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-4/9)</f>
-        <v>71.6666666666667</v>
+        <v>76.1111111111111</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A9)</f>
-        <v>58</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A9)</f>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4269,11 +4374,11 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-5/9)</f>
-        <v>57.3333333333333</v>
+        <v>60.8888888888889</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A10)</f>
-        <v>53</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A10)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4282,11 +4387,11 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-6/9)</f>
-        <v>43</v>
+        <v>45.6666666666667</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A11)</f>
-        <v>53</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4295,11 +4400,11 @@
       </c>
       <c r="B12" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-7/9)</f>
-        <v>28.6666666666667</v>
+        <v>30.4444444444444</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A12)</f>
-        <v>53</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4308,11 +4413,11 @@
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-8/9)</f>
-        <v>14.3333333333333</v>
+        <v>15.2222222222222</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A13)</f>
-        <v>53</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4324,8 +4429,8 @@
         <v>0</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$41,'Product Backlog'!$H$5:$H$41,"Hecho",'Product Backlog'!$I$5:$I$41,"&lt;="&amp;A14)</f>
-        <v>53</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: cierre del Sprint 2 con resumen, review y retrospectiva
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="291">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -476,42 +476,48 @@
     <t xml:space="preserve">Como administrador, quiero un reporte consolidado con filtros (fechas, partido, estado) e indicadores de ocupación, en PDF</t>
   </si>
   <si>
+    <t xml:space="preserve">Ocupación por partido y por sección calculada correctamente; filtros combinables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-21-reporte-admin · PR #20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /reports/reservations (JSON) y /reports/reservations/pdf: filtros opcionales y combinables (fecha de la reserva, partido, estado). Resumen por estado (todos, aunque sean 0), entradas vendidas y anuladas. Ocupación actual por partido y sección: reservas envía los asientos vendidos y match-service los cuenta con GROUP BY (endpoint interno nuevo; la lógica va donde están los datos). Capacidad = suma de secciones. Valor límite: "hasta" incluye el día completo (&lt; día siguiente 00:00). from &gt; to → 422. PDF horizontal con tarjetas y barras de ocupación (tabla de 2 celdas; casos 0 % y 100 %), tonos azules por nivel. JSON y PDF salen de la misma función (consistencia). Sin match-service → reporte con ocupación no disponible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como equipo, quiero que Reservas consulte a Partidos y valide el token por REST para mantener la integridad entre servicios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comunicación entre microservicios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asiento inexistente en Partidos → 404 desde Reservas; Partidos caído → error controlado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation-service (8083, reservation_db) valida el JWT de auth-service sin llamarlo (mismo secreto) y GET /me. match-service exige JWT de ADMIN para escribir y expone POST /internal/seats/validate con X-Internal-Key (MessageDigest.isEqual). RestClient con timeouts 2 s/3 s: 404 se propaga, caída → 503 sin guardar nada y recuperación al volver. Bug de contrato: X-Internal-Key declarado como esquema de seguridad no llegaba como header en Apidog → parámetro de header.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuario, quiero pantallas de inicio de sesión y registro para acceder al sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocupación por partido y por sección calculada correctamente; filtros combinables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como equipo, quiero que Reservas consulte a Partidos y valide el token por REST para mantener la integridad entre servicios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integración</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comunicación entre microservicios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asiento inexistente en Partidos → 404 desde Reservas; Partidos caído → error controlado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reservation-service (8083, reservation_db) valida el JWT de auth-service sin llamarlo (mismo secreto) y GET /me. match-service exige JWT de ADMIN para escribir y expone POST /internal/seats/validate con X-Internal-Key (MessageDigest.isEqual). RestClient con timeouts 2 s/3 s: 404 se propaga, caída → 503 sin guardar nada y recuperación al volver. Bug de contrato: X-Internal-Key declarado como esquema de seguridad no llegaba como header en Apidog → parámetro de header.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como usuario, quiero pantallas de inicio de sesión y registro para acceder al sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Acceso a la aplicación web (2)</t>
   </si>
   <si>
@@ -638,7 +644,10 @@
     <t xml:space="preserve">Login, cancelación y cambios de estado quedan registrados con usuario, acción y fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">Should. Recortable: si no alcanza el tiempo, se documenta como trabajo futuro (decisión de alcance del Sprint 2, replanificado el 21-oct).</t>
+    <t xml:space="preserve">Directo a main, sin PR (desviación documentada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">audit_log en auth_db y reservation_db (cada servicio en su base). AuditWriter con REQUIRES_NEW: el registro sobrevive al rollback (login con cuenta bloqueada → 423). AuditService sin transacción: nunca tumba el negocio (probado renombrando la tabla). Usuario del SecurityContext o SISTEMA; IP de la petición; solo inserción. Auditado: login éxito/fallo con motivo, bloqueo, cambio de contraseña, estados de usuario y rol, reservas creadas/confirmadas/canceladas/expiradas, reportes generados con filtros y descargas de entradas (auditoría por riesgo, no cada consulta). Bug: script no idempotente sin DROP de audit_log.</t>
   </si>
   <si>
     <t xml:space="preserve">HU-35</t>
@@ -772,6 +781,15 @@
   </si>
   <si>
     <t xml:space="preserve">Reservas con regla de 6, expiración, QR y reportes PDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incremento: reservation-service completo (disponibilidad, reservar con máximo 6, expiración automática, confirmar con tickets QR, cancelar, mis reservas, entradas y reporte del administrador en JSON y PDF), integrado con match-service (endpoints internos con X-Internal-Key) y con el JWT, más auditoría (audit_log) en auth y reservas: tríada AAA completa. 43/43 puntos. 13 bugs y hallazgos documentados (LazyInitializationException, auto-invocación transaccional, contrato del header, configuración ignorada, script no idempotente, huecos funcionales). Resumen completo en docs/sprints/sprint-2.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salió bien: se terminaron todas las historias comprometidas; fue interesante, en especial entender los PDF.
+Costó: llevó más tiempo del planificado (un día más y nuevas historias descubiertas al probar).
+Acción de mejora: probar apenas compila y tras cada arreglo; un commit por parte; revisar el servicio de cada carpeta al importar en Apidog.
+Ánimo: muchas ganas de empezar el frontend.</t>
   </si>
   <si>
     <t xml:space="preserve">Aplicación web completa para Cliente y Administrador</t>
@@ -1593,19 +1611,19 @@
                   <c:v>66</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>58</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>58</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>58</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>58</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1620,11 +1638,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="87482277"/>
-        <c:axId val="88605805"/>
+        <c:axId val="92356753"/>
+        <c:axId val="38576325"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87482277"/>
+        <c:axId val="92356753"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1690,7 +1708,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88605805"/>
+        <c:crossAx val="38576325"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1698,7 +1716,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88605805"/>
+        <c:axId val="38576325"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1774,7 +1792,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87482277"/>
+        <c:crossAx val="92356753"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2102,7 +2120,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2111,7 +2129,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.576642335766423</v>
+        <v>0.635036496350365</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2120,7 +2138,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,7 +3071,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="217.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
         <v>147</v>
       </c>
@@ -3076,30 +3094,36 @@
         <v>116</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="I25" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>46317</v>
+      </c>
       <c r="J25" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K25" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L25" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
+      <c r="M25" s="15" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>33</v>
@@ -3117,30 +3141,30 @@
         <v>46316</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>119</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>33</v>
@@ -3149,33 +3173,33 @@
         <v>3</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>33</v>
@@ -3184,33 +3208,33 @@
         <v>3</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>33</v>
@@ -3219,33 +3243,33 @@
         <v>8</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>33</v>
@@ -3254,33 +3278,33 @@
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>33</v>
@@ -3289,33 +3313,33 @@
         <v>2</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>33</v>
@@ -3324,33 +3348,33 @@
         <v>5</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>33</v>
@@ -3359,62 +3383,62 @@
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3429,27 +3453,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3464,62 +3488,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>186</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
-    <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3528,7 +3552,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3537,26 +3561,30 @@
         <v>116</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="I38" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I38" s="14" t="n">
+        <v>46317</v>
+      </c>
       <c r="J38" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="L38" s="15"/>
+        <v>204</v>
+      </c>
+      <c r="L38" s="15" t="s">
+        <v>205</v>
+      </c>
       <c r="M38" s="15" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3565,33 +3593,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3600,35 +3628,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3637,7 +3665,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3655,21 +3683,21 @@
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="M41" s="15" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>66</v>
@@ -3684,58 +3712,58 @@
         <v>5</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I42" s="14"/>
       <c r="J42" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="L42" s="15"/>
       <c r="M42" s="15" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -3796,12 +3824,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3809,34 +3837,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,7 +3872,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3853,7 +3881,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
@@ -3872,10 +3900,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3883,7 +3911,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3892,7 +3920,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
@@ -3911,18 +3939,18 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3931,7 +3959,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
@@ -3943,21 +3971,25 @@
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A7,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
-        <v>0.813953488372093</v>
-      </c>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
+        <v>1</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>46318</v>
@@ -3966,7 +3998,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
@@ -3989,10 +4021,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4001,7 +4033,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
@@ -4024,7 +4056,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4036,11 +4068,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.576642335766423</v>
+        <v>0.635036496350365</v>
       </c>
     </row>
   </sheetData>
@@ -4070,171 +4102,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4243,7 +4275,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4252,7 +4284,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4284,23 +4316,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4378,7 +4410,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A10)</f>
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4391,7 +4423,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4404,7 +4436,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4417,7 +4449,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4430,7 +4462,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gestion): HU-38 terminada e inicio del Sprint 3
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="292">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -698,7 +698,10 @@
     <t xml:space="preserve">Sección guarda x, y, ancho y alto en % del plano (0–100); fuera del plano → 400; superpuesta con otra sección → 422; GET /stadiums/{id}/layout devuelve secciones con su recuadro, filas y asientos; semillas con coordenadas</t>
   </si>
   <si>
-    <t xml:space="preserve">Idea de la usuaria (22-oct): al crear secciones, ubicarlas como recuadros sobre el plano, porque un enum de lado (norte/sur/...) no representa estadios reales. Geometría en porcentaje para que el mapa escale a cualquier pantalla. Incluye el endpoint /layout pendiente desde HU-07. Requisito del mapa de asientos del frontend. Primero: formulario con vista previa en vivo.</t>
+    <t xml:space="preserve">feature/HU-38-plano-estadio · PR #22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuadro de cada sección (x, y, ancho, alto en % del plano, enteros) como @Embeddable SectionBox con overlaps(): no pisa la cancha (fija, x 28 y 25 44×50) ni otra sección → 422; tocarse en el borde no es superponerse (valor límite). Validación cruzada @AssertTrue isInsidePlan → 400. PUT /sections/{id}/box (se ignora a sí misma al mover) y box opcional al crear. Base: columnas pos_x, pos_y, width, height con CHECK de completitud y de plano (+4 pruebas, 24/24), semillas ubicadas. GET /stadiums/{id}/layout público: cancha, recuadros, filas y asientos, sin disponibilidad (estático vs. dinámico); N+1 con batch fetch. Bugs: base desactualizada → validate impidió arrancar y respondía la instancia vieja; dependencia circular SectionService → sí mismo; springdoc dentro de spring: (ignorado desde el Sprint 1).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-39</t>
@@ -1611,19 +1614,19 @@
                   <c:v>66</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>50</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>50</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>50</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>50</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1638,11 +1641,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="92356753"/>
-        <c:axId val="38576325"/>
+        <c:axId val="71162524"/>
+        <c:axId val="22290464"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92356753"/>
+        <c:axId val="71162524"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1708,7 +1711,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38576325"/>
+        <c:crossAx val="22290464"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1716,7 +1719,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38576325"/>
+        <c:axId val="22290464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1792,7 +1795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92356753"/>
+        <c:crossAx val="71162524"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2120,7 +2123,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2129,7 +2132,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.635036496350365</v>
+        <v>0.671532846715328</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2138,7 +2141,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3692,7 +3695,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
         <v>220</v>
       </c>
@@ -3715,26 +3718,30 @@
         <v>161</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="I42" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I42" s="14" t="n">
+        <v>46317</v>
+      </c>
       <c r="J42" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="L42" s="15"/>
+      <c r="L42" s="15" t="s">
+        <v>223</v>
+      </c>
       <c r="M42" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
@@ -3759,11 +3766,11 @@
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -3824,12 +3831,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3837,34 +3844,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,7 +3879,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3881,7 +3888,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
@@ -3900,10 +3907,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3911,7 +3918,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3920,7 +3927,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
@@ -3939,10 +3946,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3950,7 +3957,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3959,7 +3966,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
@@ -3978,10 +3985,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3992,13 +3999,13 @@
         <v>160</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
@@ -4010,11 +4017,11 @@
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">IF(G8=0,0,H8/G8)</f>
-        <v>0</v>
+        <v>0.161290322580645</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
@@ -4024,7 +4031,7 @@
         <v>189</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4033,7 +4040,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
@@ -4056,7 +4063,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4068,11 +4075,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.635036496350365</v>
+        <v>0.671532846715328</v>
       </c>
     </row>
   </sheetData>
@@ -4102,104 +4109,104 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
@@ -4210,63 +4217,63 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4275,7 +4282,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4284,7 +4291,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4316,23 +4323,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4410,7 +4417,7 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A10)</f>
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4423,7 +4430,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4436,7 +4443,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4449,7 +4456,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4462,7 +4469,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gestion): HU-29 y HU-24 terminadas
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="298">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -533,18 +533,24 @@
     <t xml:space="preserve">Como cliente, quiero un catálogo de partidos con búsqueda por fecha para elegir un evento</t>
   </si>
   <si>
+    <t xml:space="preserve">Búsqueda por fecha funciona; muestra estadio, fecha y hora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-24-catalogo · PR #27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catálogo público en /: por defecto PROGRAMADO desde hoy; búsqueda por fecha y por equipo (mínimo 2 letras, validado antes de llamar). Endpoints públicos sin token (un token vencido no causa 401). Respuestas viejas ignoradas (race condition). Fechas con Intl es-EC armadas en hora local (new Date("AAAA-MM-DD") las corre un día por UTC). Cuatro estados: cargando, error, vacío y con datos. Bug: rutas nuevas fuera del Layout y "/" duplicada → seguía la página vieja.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero un mapa gráfico de asientos por sección y fila con disponibilidad en tiempo real para elegir mis asientos</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Búsqueda por fecha funciona; muestra estadio, fecha y hora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero un mapa gráfico de asientos por sección y fila con disponibilidad en tiempo real para elegir mis asientos</t>
-  </si>
-  <si>
     <t xml:space="preserve">Usabilidad y experiencia de usuario (5)</t>
   </si>
   <si>
@@ -588,6 +594,12 @@
   </si>
   <si>
     <t xml:space="preserve">Cliente no ve menú admin; URL admin sin permiso redirige</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-29-menu-por-rol · PR #26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menú según el rol (público, CLIENTE, ADMIN) y rutas agrupadas con ProtectedRoute + &lt;Outlet/&gt;: sin sesión → login y vuelve a la página pedida; rol ajeno → acceso denegado; mustChangePassword → siempre al cambio de contraseña (en el Layout). Aviso de sesión vencida tras un 401. No es seguridad (el backend responde 401/403): defensa en profundidad comprobada en Apidog. Menú del usuario con &lt;details&gt; nativo. Bugs: CSS del navbar no aplicado; el menú quedaba abierto al navegar (useRef).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-30</t>
@@ -1623,16 +1635,16 @@
                   <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>42</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>42</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>42</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>42</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1647,11 +1659,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="93490531"/>
-        <c:axId val="23560430"/>
+        <c:axId val="94338474"/>
+        <c:axId val="75185692"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="93490531"/>
+        <c:axId val="94338474"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1717,7 +1729,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23560430"/>
+        <c:crossAx val="75185692"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1725,7 +1737,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23560430"/>
+        <c:axId val="75185692"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1801,7 +1813,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93490531"/>
+        <c:crossAx val="94338474"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2129,7 +2141,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2138,7 +2150,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.693430656934307</v>
+        <v>0.72992700729927</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2147,7 +2159,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,7 +3215,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
         <v>166</v>
       </c>
@@ -3226,24 +3238,30 @@
         <v>161</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="I28" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>46318</v>
+      </c>
       <c r="J28" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K28" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="L28" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
+      <c r="M28" s="15" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
@@ -3261,24 +3279,24 @@
         <v>161</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
@@ -3296,24 +3314,24 @@
         <v>161</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
@@ -3331,24 +3349,24 @@
         <v>161</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
@@ -3366,24 +3384,24 @@
         <v>161</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
-    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
@@ -3401,59 +3419,65 @@
         <v>161</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="I33" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I33" s="14" t="n">
+        <v>46318</v>
+      </c>
       <c r="J33" s="5" t="s">
         <v>162</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
+        <v>188</v>
+      </c>
+      <c r="L33" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="M33" s="15" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3468,27 +3492,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3503,62 +3527,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3567,7 +3591,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3585,21 +3609,21 @@
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="L38" s="15" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="M38" s="15" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3608,33 +3632,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3643,35 +3667,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3680,7 +3704,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3698,21 +3722,21 @@
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="M41" s="15" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>66</v>
@@ -3739,21 +3763,21 @@
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="L42" s="15" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="M42" s="15" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
@@ -3762,27 +3786,27 @@
         <v>160</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -3843,12 +3867,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3856,34 +3880,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3891,7 +3915,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3900,7 +3924,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
@@ -3919,10 +3943,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,7 +3954,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3939,7 +3963,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
@@ -3958,10 +3982,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,7 +3993,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -3978,7 +4002,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
@@ -3997,10 +4021,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,7 +4041,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
@@ -4029,21 +4053,21 @@
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">IF(G8=0,0,H8/G8)</f>
-        <v>0.258064516129032</v>
+        <v>0.419354838709677</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4052,7 +4076,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
@@ -4075,7 +4099,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4087,11 +4111,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.693430656934307</v>
+        <v>0.72992700729927</v>
       </c>
     </row>
   </sheetData>
@@ -4121,171 +4145,171 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4294,7 +4318,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4303,7 +4327,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4335,23 +4359,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4442,7 +4466,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4455,7 +4479,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4468,7 +4492,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4481,7 +4505,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gestion): HU-25, HU-26 y HU-27 terminadas
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="302">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -548,37 +548,49 @@
     <t xml:space="preserve">Como cliente, quiero un mapa gráfico de asientos por sección y fila con disponibilidad en tiempo real para elegir mis asientos</t>
   </si>
   <si>
+    <t xml:space="preserve">Usabilidad y experiencia de usuario (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colores libre/ocupado/seleccionado con leyenda; se actualiza sin recargar; no deja elegir más de 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-25-mapa-asientos · PR #28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano SVG del estadio (lienzo cuadrado: cancha vertical con áreas, arcos y pista; secciones en sus recuadros con nombre ajustado a 1-2 líneas) y grilla de asientos orientada hacia la cancha (la fila A siempre pegada a la cancha, CSS Grid). Estructura una vez + disponibilidad cada refreshSeconds, pausada si la pestaña no está visible (usePolling, sin fugas). Índice seatId → asiento. Si otro cliente toma un asiento elegido, se quita de la selección y se avisa. Disponibilidad pública en el backend (solo ids). Accesible con teclado y sin depender solo del color. Bugs: archivos editados en otra carpeta / zip fuera del proyecto; CSS y JSX de versiones distintas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero un formulario de confirmación de reserva (máximo 6) para cerrar mi compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen antes de confirmar; error 409/422 mostrado en lenguaje claro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar desde el mapa (botón desactivado mientras responde; 409 recarga la disponibilidad) y pantalla de la reserva con cuenta regresiva: la hora sin zona del backend se interpreta con -05:00 (Ecuador no tiene horario de verano), así funciona en cualquier zona horaria; ámbar en el último minuto y aviso al vencer. Confirmar y cancelar en dos pasos (botón secundario rojo). Hallazgo: commit mal etiquetado con archivos Java copiados dentro de frontend/src (eliminados y documentado en el PR). Mejora futura: cancelar por asiento (HU-36).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como cliente, quiero ver mi boleto electrónico con código QR para presentarlo en el ingreso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QR visible y legible por un lector de celular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entradas con su QR en pantalla: la imagen requiere token, así que se descarga como Blob y se muestra con una URL temporal que se libera al salir (sin fugas de memoria). Descarga del PDF de entradas. Tickets anulados sin QR. QR escaneado con el celular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quiero pantallas de usuarios/roles, estadios, partidos, reservas por evento y reporte general</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usabilidad y experiencia de usuario (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colores libre/ocupado/seleccionado con leyenda; se actualiza sin recargar; no deja elegir más de 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero un formulario de confirmación de reserva (máximo 6) para cerrar mi compra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumen antes de confirmar; error 409/422 mostrado en lenguaje claro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como cliente, quiero ver mi boleto electrónico con código QR para presentarlo en el ingreso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QR visible y legible por un lector de celular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quiero pantallas de usuarios/roles, estadios, partidos, reservas por evento y reporte general</t>
   </si>
   <si>
     <t xml:space="preserve">Consumo de microservicios desde la interfaz (5)</t>
@@ -1635,16 +1647,16 @@
                   <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>37</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>37</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>37</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>37</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1659,11 +1671,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94338474"/>
-        <c:axId val="75185692"/>
+        <c:axId val="64712088"/>
+        <c:axId val="85719523"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94338474"/>
+        <c:axId val="64712088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1729,7 +1741,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75185692"/>
+        <c:crossAx val="85719523"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1737,7 +1749,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75185692"/>
+        <c:axId val="85719523"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1813,7 +1825,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94338474"/>
+        <c:crossAx val="64712088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2141,7 +2153,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2150,7 +2162,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.72992700729927</v>
+        <v>0.824817518248175</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2159,7 +2171,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3256,7 +3268,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
         <v>171</v>
       </c>
@@ -3279,24 +3291,30 @@
         <v>161</v>
       </c>
       <c r="H29" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I29" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="J29" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="I29" s="14"/>
-      <c r="J29" s="5" t="s">
+      <c r="K29" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="K29" s="5" t="s">
+      <c r="L29" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-    </row>
-    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M29" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>66</v>
@@ -3314,24 +3332,30 @@
         <v>161</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="I30" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I30" s="14" t="n">
+        <v>46318</v>
+      </c>
       <c r="J30" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-    </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>179</v>
+      </c>
+      <c r="L30" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="M30" s="15" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>66</v>
@@ -3349,24 +3373,30 @@
         <v>161</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="I31" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="I31" s="14" t="n">
+        <v>46318</v>
+      </c>
       <c r="J31" s="5" t="s">
         <v>133</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
+        <v>183</v>
+      </c>
+      <c r="L31" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="M31" s="15" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>66</v>
@@ -3384,24 +3414,24 @@
         <v>161</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="5" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
@@ -3428,56 +3458,56 @@
         <v>162</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="L33" s="15" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3492,27 +3522,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3527,62 +3557,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3591,7 +3621,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3609,21 +3639,21 @@
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="L38" s="15" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="M38" s="15" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3632,33 +3662,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3667,35 +3697,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3704,7 +3734,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3722,21 +3752,21 @@
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="M41" s="15" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>66</v>
@@ -3763,21 +3793,21 @@
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="L42" s="15" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="M42" s="15" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
@@ -3786,27 +3816,27 @@
         <v>160</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -3867,12 +3897,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3880,34 +3910,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3915,7 +3945,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3924,7 +3954,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
@@ -3943,10 +3973,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3954,7 +3984,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3963,7 +3993,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
@@ -3982,10 +4012,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3993,7 +4023,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -4002,7 +4032,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
@@ -4021,10 +4051,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4041,7 +4071,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
@@ -4053,21 +4083,21 @@
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">IF(G8=0,0,H8/G8)</f>
-        <v>0.419354838709677</v>
+        <v>0.838709677419355</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4076,7 +4106,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
@@ -4099,7 +4129,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4111,11 +4141,11 @@
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.72992700729927</v>
+        <v>0.824817518248175</v>
       </c>
     </row>
   </sheetData>
@@ -4145,104 +4175,104 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
@@ -4253,63 +4283,63 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4318,7 +4348,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4327,7 +4357,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4359,23 +4389,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4466,7 +4496,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4479,7 +4509,7 @@
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4492,7 +4522,7 @@
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4505,7 +4535,7 @@
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(gestion): HU-20 front terminada, HU-28 en curso
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="305">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -464,10 +464,10 @@
     <t xml:space="preserve">Solo muestra reservas propias; PDF se genera y abre</t>
   </si>
   <si>
-    <t xml:space="preserve">feature/HU-20-mis-reservas-pdf · PR #18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GET /reservations/me (JSON) y /me/pdf (OpenPDF): historial del cliente del token (seguridad por diseño: no recibe id), de la más nueva a la más antigua. Datos del partido pedidos a match-service una vez por partido distinto, fuera de la transacción; si no responde → match null / "información no disponible" (degradación elegante). N+1 local resuelto con default_batch_fetch_size (bug de configuración: estaba bajo spring.jpa.hibernate y se ignoraba sin error). ADMIN → 403. Limitación del modelo: reservas canceladas/expiradas sin confirmar no conservan sus asientos (seat_lock es el candado vigente, no historial). Hallazgos Sonar: throws Exception sobrante, CSRF documentado (S4502), literales de rol (S1192).</t>
+    <t xml:space="preserve">feature/HU-20-mis-reservas-pdf · PR #18 · feature/HU-20-mis-reservas-frontend · PR #29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Front (PR #29, 23-oct): pantalla /reservas con filtros Activas/Historial/Todas (en el cliente), PENDIENTE vencida mostrada como EXPIRADA, descarga del PDF, estado vacío y "Partido #id" si match-service cae. Back: GET /reservations/me (JSON) y /me/pdf (OpenPDF): historial del cliente del token (seguridad por diseño: no recibe id), de la más nueva a la más antigua. Datos del partido pedidos a match-service una vez por partido distinto, fuera de la transacción; si no responde → match null / "información no disponible" (degradación elegante). N+1 local resuelto con default_batch_fetch_size (bug de configuración: estaba bajo spring.jpa.hibernate y se ignoraba sin error). ADMIN → 403. Limitación del modelo: reservas canceladas/expiradas sin confirmar no conservan sus asientos (seat_lock es el candado vigente, no historial). Hallazgos Sonar: throws Exception sobrante, CSRF documentado (S4502), literales de rol (S1192).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-21</t>
@@ -590,43 +590,52 @@
     <t xml:space="preserve">Como administrador, quiero pantallas de usuarios/roles, estadios, partidos, reservas por evento y reporte general</t>
   </si>
   <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consumo de microservicios desde la interfaz (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada pantalla consume su microservicio; operaciones CRUD visibles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-28-admin-estadios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parte 1 (23-oct): estadios (listar, crear, editar, eliminar con confirmación; 409 si tiene secciones o partidos) y secciones + plano (crear sección con capacidad disponible en vivo; ubicar/mover recuadro con vista previa en el mapa y las mismas reglas del backend: límites, cancha y superposición). Faltan: partidos, usuarios/roles y reportes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como usuario, quiero ver solo las opciones de mi rol para no acceder a funciones ajenas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliente no ve menú admin; URL admin sin permiso redirige</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feature/HU-29-menu-por-rol · PR #26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menú según el rol (público, CLIENTE, ADMIN) y rutas agrupadas con ProtectedRoute + &lt;Outlet/&gt;: sin sesión → login y vuelve a la página pedida; rol ajeno → acceso denegado; mustChangePassword → siempre al cambio de contraseña (en el Layout). Aviso de sesión vencida tras un 401. No es seguridad (el backend responde 401/403): defensa en profundidad comprobada en Apidog. Menú del usuario con &lt;details&gt; nativo. Bugs: CSS del navbar no aplicado; el menú quedaba abierto al navegar (useRef).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como QA, quiero pruebas E2E en Apidog de las reglas de negocio para demostrar que el sistema funciona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consumo de microservicios desde la interfaz (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cada pantalla consume su microservicio; operaciones CRUD visibles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como usuario, quiero ver solo las opciones de mi rol para no acceder a funciones ajenas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cliente no ve menú admin; URL admin sin permiso redirige</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feature/HU-29-menu-por-rol · PR #26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menú según el rol (público, CLIENTE, ADMIN) y rutas agrupadas con ProtectedRoute + &lt;Outlet/&gt;: sin sesión → login y vuelve a la página pedida; rol ajeno → acceso denegado; mustChangePassword → siempre al cambio de contraseña (en el Layout). Aviso de sesión vencida tras un 401. No es seguridad (el backend responde 401/403): defensa en profundidad comprobada en Apidog. Menú del usuario con &lt;details&gt; nativo. Bugs: CSS del navbar no aplicado; el menú quedaba abierto al navegar (useRef).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HU-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como QA, quiero pruebas E2E en Apidog de las reglas de negocio para demostrar que el sistema funciona</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 4</t>
   </si>
   <si>
     <t xml:space="preserve">Defensa</t>
@@ -1214,7 +1223,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1258,6 +1267,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1671,11 +1688,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="64712088"/>
-        <c:axId val="85719523"/>
+        <c:axId val="62658198"/>
+        <c:axId val="62674309"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="64712088"/>
+        <c:axId val="62658198"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1741,7 +1758,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85719523"/>
+        <c:crossAx val="62674309"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1749,7 +1766,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85719523"/>
+        <c:axId val="62674309"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1825,7 +1842,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64712088"/>
+        <c:crossAx val="62658198"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3063,7 +3080,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="204.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="267.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
         <v>141</v>
       </c>
@@ -3391,7 +3408,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
         <v>185</v>
       </c>
@@ -3423,15 +3440,19 @@
       <c r="K32" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
+      <c r="L32" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="M32" s="15" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
@@ -3458,56 +3479,56 @@
         <v>162</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="L33" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3522,27 +3543,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3557,62 +3578,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>200</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>198</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3621,7 +3642,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3639,21 +3660,21 @@
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="L38" s="15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="M38" s="15" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3662,33 +3683,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3697,35 +3718,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3734,7 +3755,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3752,21 +3773,21 @@
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="M41" s="15" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>66</v>
@@ -3793,21 +3814,21 @@
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="L42" s="15" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="M42" s="15" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
@@ -3816,39 +3837,39 @@
         <v>160</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M43"/>
   <conditionalFormatting sqref="H5:H43">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3897,12 +3918,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3910,34 +3931,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3945,7 +3966,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3954,7 +3975,7 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
@@ -3973,10 +3994,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3984,7 +4005,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -3993,7 +4014,7 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
@@ -4012,10 +4033,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4023,7 +4044,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -4032,7 +4053,7 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
@@ -4051,10 +4072,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4071,7 +4092,7 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
@@ -4094,10 +4115,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4106,7 +4127,7 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
@@ -4129,7 +4150,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4175,104 +4196,104 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
@@ -4283,63 +4304,63 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4348,7 +4369,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4357,7 +4378,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4389,23 +4410,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs(gestion): HU-28 y HU-40 terminadas
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Burndown" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="308">
   <si>
     <t xml:space="preserve">Plan de Sprints — Sistema de Gestión de Entradas para Eventos Deportivos</t>
   </si>
@@ -590,19 +590,16 @@
     <t xml:space="preserve">Como administrador, quiero pantallas de usuarios/roles, estadios, partidos, reservas por evento y reporte general</t>
   </si>
   <si>
-    <t xml:space="preserve">En curso</t>
-  </si>
-  <si>
     <t xml:space="preserve">Consumo de microservicios desde la interfaz (5)</t>
   </si>
   <si>
     <t xml:space="preserve">Cada pantalla consume su microservicio; operaciones CRUD visibles</t>
   </si>
   <si>
-    <t xml:space="preserve">feature/HU-28-admin-estadios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parte 1 (23-oct): estadios (listar, crear, editar, eliminar con confirmación; 409 si tiene secciones o partidos) y secciones + plano (crear sección con capacidad disponible en vivo; ubicar/mover recuadro con vista previa en el mapa y las mismas reglas del backend: límites, cancha y superposición). Faltan: partidos, usuarios/roles y reportes.</t>
+    <t xml:space="preserve">feature/HU-28-admin-estadios · PR #30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel del admin completo: estadios (CRUD, 409 si tiene secciones o partidos) y secciones con plano (vista previa en el mapa reutilizando StadiumMap, mismas reglas que el backend: límites, cancha, superposición); partidos con máquina de estados (solo botones válidos, confirmación en finalizar/cancelar, estadio fijo al editar); usuarios y roles (activar, desactivar, desbloquear; no se desactiva a sí mismo ni a ADMIN); reportes (KPIs, ocupación por partido y sección, PDF con los mismos filtros) y reservas por evento con cancelación por el admin (clientId solo en DTO de admin). Hallazgos de QA al probar: nombres únicos ignoraban tildes (índice con name_key + unaccent), registro con rol CLIENTE inactivo daba 500 (ahora 422), secciones grandes ilegibles (bloques), semillas con tamaños reales (8 460 asientos por estadio). Limitación: desactivar no corta un JWT vigente (60 min).</t>
   </si>
   <si>
     <t xml:space="preserve">HU-29</t>
@@ -753,6 +750,18 @@
   </si>
   <si>
     <t xml:space="preserve">Mejora visual de HU-38: editor de arrastrar y soltar (por ejemplo react-rnd). Recortable: HU-38 ya permite ubicar las secciones con números y vista previa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como negocio, quiero que la venta online cierre a una hora fija respecto del inicio del partido, aunque el admin no cambie el estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar o confirmar después de inicio + SALES_CLOSE_OFFSET_MINUTES → 422; la reserva vence a más tardar al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regla nueva propuesta al probar HU-28: el estado lo cambia una persona, la hora es un hecho. SalesWindow (único dueño de la regla) en reservar, confirmar y disponibilidad: PROGRAMADO o EN_CURSO y antes de inicio + SALES_CLOSE_OFFSET_MINUTES (10, configurable; negativo = antes). expiresAt = min(ahora + HOLD_MINUTES, cierre). match-service envía fecha y hora en la validación de asientos (una sola llamada). El front solo lee salesOpen/salesCloseAt: no se calcula con el reloj del cliente.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprints</t>
@@ -1223,7 +1232,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1267,14 +1276,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1514,31 +1515,31 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>137</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>121.777777777778</c:v>
+                  <c:v>124.444444444444</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>106.555555555556</c:v>
+                  <c:v>108.888888888889</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>91.3333333333333</c:v>
+                  <c:v>93.3333333333333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>76.1111111111111</c:v>
+                  <c:v>77.7777777777778</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>60.8888888888889</c:v>
+                  <c:v>62.2222222222222</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>45.6666666666667</c:v>
+                  <c:v>46.6666666666667</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>30.4444444444444</c:v>
+                  <c:v>31.1111111111111</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15.2222222222222</c:v>
+                  <c:v>15.5555555555556</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1646,34 +1647,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>124</c:v>
+                  <c:v>127</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>115</c:v>
+                  <c:v>118</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>109</c:v>
+                  <c:v>112</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>93</c:v>
+                  <c:v>96</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>66</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>24</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>24</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>24</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>24</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1688,11 +1689,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62658198"/>
-        <c:axId val="62674309"/>
+        <c:axId val="2604376"/>
+        <c:axId val="76982257"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62658198"/>
+        <c:axId val="2604376"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1758,7 +1759,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62674309"/>
+        <c:crossAx val="76982257"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1766,7 +1767,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62674309"/>
+        <c:axId val="76982257"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1842,7 +1843,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62658198"/>
+        <c:crossAx val="2604376"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2151,8 +2152,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTA('Product Backlog'!A5:A43)</f>
-        <v>39</v>
+        <f aca="false">COUNTA('Product Backlog'!A5:A44)</f>
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2160,8 +2161,8 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">SUM('Product Backlog'!F5:F43)</f>
-        <v>137</v>
+        <f aca="false">SUM('Product Backlog'!F5:F44)</f>
+        <v>140</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2169,8 +2170,8 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!F5:F43,'Product Backlog'!H5:H43,"Hecho")</f>
-        <v>113</v>
+        <f aca="false">SUMIFS('Product Backlog'!F5:F44,'Product Backlog'!H5:H44,"Hecho")</f>
+        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2179,7 +2180,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IF(B7=0,0,B8/B7)</f>
-        <v>0.824817518248175</v>
+        <v>0.864285714285714</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2187,8 +2188,8 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!H5:H43,"Hecho")</f>
-        <v>31</v>
+        <f aca="false">COUNTIF('Product Backlog'!H5:H44,"Hecho")</f>
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2232,7 +2233,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3408,7 +3409,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="255.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
         <v>185</v>
       </c>
@@ -3431,28 +3432,30 @@
         <v>161</v>
       </c>
       <c r="H32" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="J32" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="I32" s="14"/>
-      <c r="J32" s="5" t="s">
+      <c r="K32" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="K32" s="5" t="s">
+      <c r="L32" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="L32" s="15" t="s">
+      <c r="M32" s="15" t="s">
         <v>190</v>
-      </c>
-      <c r="M32" s="15" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>66</v>
@@ -3479,56 +3482,56 @@
         <v>162</v>
       </c>
       <c r="K33" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="L33" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="L33" s="15" t="s">
+      <c r="M33" s="15" t="s">
         <v>195</v>
-      </c>
-      <c r="M33" s="15" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>198</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E34" s="11" t="s">
         <v>199</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>200</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H34" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="K34" s="5" t="s">
         <v>203</v>
-      </c>
-      <c r="K34" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>31</v>
@@ -3543,27 +3546,27 @@
         <v>3</v>
       </c>
       <c r="G35" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H35" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H35" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>209</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>31</v>
@@ -3578,62 +3581,62 @@
         <v>2</v>
       </c>
       <c r="G36" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H36" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H36" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="K36" s="5" t="s">
         <v>210</v>
-      </c>
-      <c r="K36" s="5" t="s">
-        <v>211</v>
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>212</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>213</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G37" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H37" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H37" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I37" s="14"/>
       <c r="J37" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>31</v>
@@ -3642,7 +3645,7 @@
         <v>90</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F38" s="12" t="n">
         <v>3</v>
@@ -3660,21 +3663,21 @@
         <v>91</v>
       </c>
       <c r="K38" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="L38" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="L38" s="15" t="s">
+      <c r="M38" s="15" t="s">
         <v>218</v>
-      </c>
-      <c r="M38" s="15" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>221</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>31</v>
@@ -3683,33 +3686,33 @@
         <v>115</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G39" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H39" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H39" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>225</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>66</v>
@@ -3718,35 +3721,35 @@
         <v>115</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F40" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H40" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H40" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="5" t="s">
         <v>117</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>228</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>229</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>66</v>
@@ -3755,7 +3758,7 @@
         <v>115</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>3</v>
@@ -3773,21 +3776,21 @@
         <v>133</v>
       </c>
       <c r="K41" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="L41" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="L41" s="15" t="s">
+      <c r="M41" s="15" t="s">
         <v>231</v>
-      </c>
-      <c r="M41" s="15" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="242.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>233</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>234</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>66</v>
@@ -3814,21 +3817,21 @@
         <v>143</v>
       </c>
       <c r="K42" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="L42" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="L42" s="15" t="s">
+      <c r="M42" s="15" t="s">
         <v>236</v>
-      </c>
-      <c r="M42" s="15" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B43" s="5" t="s">
         <v>238</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>239</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>66</v>
@@ -3837,52 +3840,93 @@
         <v>160</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="H43" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="H43" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="5" t="s">
         <v>143</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10" t="s">
         <v>241</v>
       </c>
+      <c r="B44" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="F44" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="H44" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I44" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K44" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="L44" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="M44" s="15" t="s">
+        <v>244</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M43"/>
-  <conditionalFormatting sqref="H5:H43">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+  <autoFilter ref="A4:M44"/>
+  <conditionalFormatting sqref="H5:H44">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Hecho"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"En curso"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H43" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
       <formula1>"Pendiente,En curso,Hecho,Bloqueado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G44" type="list">
       <formula1>Sprints!$A$5:$A$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I43" type="date">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I44" type="date">
       <formula1>DATE(2026,10,17)</formula1>
       <formula2>DATE(2026,10,26)</formula2>
     </dataValidation>
@@ -3918,12 +3962,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3931,34 +3975,34 @@
         <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3966,7 +4010,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>46312</v>
@@ -3975,18 +4019,18 @@
         <v>46312</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$44,A5)</f>
         <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A5)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A5)</f>
         <v>13</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A5,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A5,'Product Backlog'!$H$5:$H$44,"Hecho")</f>
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
@@ -3994,10 +4038,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4005,7 +4049,7 @@
         <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>46313</v>
@@ -4014,18 +4058,18 @@
         <v>46315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$44,A6)</f>
         <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A6)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A6)</f>
         <v>31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A6,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A6,'Product Backlog'!$H$5:$H$44,"Hecho")</f>
         <v>31</v>
       </c>
       <c r="I6" s="6" t="n">
@@ -4033,10 +4077,10 @@
         <v>1</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="229.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4044,7 +4088,7 @@
         <v>116</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>46315</v>
@@ -4053,18 +4097,18 @@
         <v>46317</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$44,A7)</f>
         <v>10</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A7)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A7)</f>
         <v>43</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A7,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A7,'Product Backlog'!$H$5:$H$44,"Hecho")</f>
         <v>43</v>
       </c>
       <c r="I7" s="6" t="n">
@@ -4072,10 +4116,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4092,33 +4136,33 @@
         <v>46319</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A8)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$44,A8)</f>
+        <v>9</v>
       </c>
       <c r="G8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8)</f>
-        <v>31</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A8)</f>
+        <v>34</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A8,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
-        <v>26</v>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A8,'Product Backlog'!$H$5:$H$44,"Hecho")</f>
+        <v>34</v>
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">IF(G8=0,0,H8/G8)</f>
-        <v>0.838709677419355</v>
+        <v>1</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>46320</v>
@@ -4127,18 +4171,18 @@
         <v>46321</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$43,A9)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$44,A9)</f>
         <v>7</v>
       </c>
       <c r="G9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A9)</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A9)</f>
         <v>19</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$G$5:$G$43,A9,'Product Backlog'!$H$5:$H$43,"Hecho")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$G$5:$G$44,A9,'Product Backlog'!$H$5:$H$44,"Hecho")</f>
         <v>0</v>
       </c>
       <c r="I9" s="6" t="n">
@@ -4150,23 +4194,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G10" s="3" t="n">
         <f aca="false">SUM(G5:G9)</f>
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
-        <v>0.824817518248175</v>
+        <v>0.864285714285714</v>
       </c>
     </row>
   </sheetData>
@@ -4196,104 +4240,104 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>5</v>
@@ -4304,63 +4348,63 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C15" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Servicios")</f>
@@ -4369,7 +4413,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C16" s="3" t="n">
         <f aca="false">SUMIFS(C5:C14,A5:A14,"Arquitectura")</f>
@@ -4378,7 +4422,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C17" s="3" t="n">
         <f aca="false">(C15+C16)/2</f>
@@ -4410,23 +4454,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4435,11 +4479,11 @@
       </c>
       <c r="B5" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-0/9)</f>
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A5)</f>
-        <v>124</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A5)</f>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4448,11 +4492,11 @@
       </c>
       <c r="B6" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-1/9)</f>
-        <v>121.777777777778</v>
+        <v>124.444444444444</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A6)</f>
-        <v>115</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A6)</f>
+        <v>118</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4461,11 +4505,11 @@
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-2/9)</f>
-        <v>106.555555555556</v>
+        <v>108.888888888889</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A7)</f>
-        <v>109</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A7)</f>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4474,11 +4518,11 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-3/9)</f>
-        <v>91.3333333333333</v>
+        <v>93.3333333333333</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A8)</f>
-        <v>93</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A8)</f>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4487,11 +4531,11 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-4/9)</f>
-        <v>76.1111111111111</v>
+        <v>77.7777777777778</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A9)</f>
-        <v>66</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A9)</f>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4500,11 +4544,11 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-5/9)</f>
-        <v>60.8888888888889</v>
+        <v>62.2222222222222</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A10)</f>
-        <v>45</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A10)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4513,11 +4557,11 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-6/9)</f>
-        <v>45.6666666666667</v>
+        <v>46.6666666666667</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A11)</f>
-        <v>24</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A11)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4526,11 +4570,11 @@
       </c>
       <c r="B12" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-7/9)</f>
-        <v>30.4444444444444</v>
+        <v>31.1111111111111</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A12)</f>
-        <v>24</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A12)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,11 +4583,11 @@
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">Resumen!$B$7*(1-8/9)</f>
-        <v>15.2222222222222</v>
+        <v>15.5555555555556</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A13)</f>
-        <v>24</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A13)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4555,8 +4599,8 @@
         <v>0</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$43,'Product Backlog'!$H$5:$H$43,"Hecho",'Product Backlog'!$I$5:$I$43,"&lt;="&amp;A14)</f>
-        <v>24</v>
+        <f aca="false">Resumen!$B$7-SUMIFS('Product Backlog'!$F$5:$F$44,'Product Backlog'!$H$5:$H$44,"Hecho",'Product Backlog'!$I$5:$I$44,"&lt;="&amp;A14)</f>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: actulizacion de docuemtos
</commit_message>
<xml_diff>
--- a/docs/gestion/Plan_Sprints_Complexivo.xlsx
+++ b/docs/gestion/Plan_Sprints_Complexivo.xlsx
@@ -1884,7 +1884,7 @@
       </c>
       <c r="M11" s="36" t="inlineStr">
         <is>
-          <t>Entidades Section/SeatRow/Seat con relaciones y cascade. GET y POST de secciones: genera filas A..Z y asientos 1..N en una transacción. 400 tipo fuera de catálogo / rangos; 404; 409 nombre por estadio; 422 si supera la capacidad del estadio. Pendiente (nueva HU): editar/eliminar sección y endpoint layout. Mejora: bloqueo pesimista para la regla de capacidad con concurrencia.</t>
+          <t>Entidades Section/SeatRow/Seat con relaciones y cascade. GET y POST de secciones: genera filas A..Z y asientos 1..N en una transacción. 400 tipo fuera de catálogo / rangos; 404; 409 nombre por estadio; 422 si supera la capacidad del estadio. Endpoint layout hecho en HU-38. 26-oct: se implementó la edición de nombre y descripción (PUT /sections/{id}) al detectar en Apidog que el contrato la documentaba sin implementación (404). Eliminar sección queda pendiente. Mejora: bloqueo pesimista para la regla de capacidad con concurrencia.</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       <c r="L34" s="36" t="n"/>
       <c r="M34" s="36" t="inlineStr">
         <is>
-          <t>56 casos E2E de API listos para Apidog (docs/pruebas/apidog). Falta ejecutarlos y registrar el resultado.</t>
+          <t>26-oct: flujo E2E ejecutado en Apidog (login cliente → reservar → confirmar → login admin → validar QR), 5 de 5 aprobados, más casos negativos. Prueba de concurrencia con k6 (docs/pruebas/k6): 50 usuarios sobre el mismo asiento → 1 reserva creada y 49 rechazadas con 409; carga de disponibilidad con 20 usuarios durante 30 s: 24 121 solicitudes, p95 37,7 ms, 0 % de errores. Pasar a Hecho cuando estén ejecutados los cuatro escenarios de los criterios.</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="I35" s="35" t="n"/>
@@ -3382,7 +3382,11 @@
         </is>
       </c>
       <c r="L35" s="36" t="n"/>
-      <c r="M35" s="36" t="n"/>
+      <c r="M35" s="36" t="inlineStr">
+        <is>
+          <t>README con instrucciones para levantar el sistema, variables de entorno y usuarios de prueba (puerto de Mailpit 2525). Faltan el .env de ejemplo y Docker Compose (trabajo futuro).</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26.85" customHeight="1" s="21">
       <c r="A36" s="31" t="inlineStr">
@@ -3420,10 +3424,12 @@
       </c>
       <c r="H36" s="34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I36" s="35" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I36" s="35" t="n">
+        <v>46321</v>
+      </c>
       <c r="J36" s="26" t="inlineStr">
         <is>
           <t>Arquitectura de software</t>
@@ -3435,7 +3441,11 @@
         </is>
       </c>
       <c r="L36" s="36" t="n"/>
-      <c r="M36" s="36" t="n"/>
+      <c r="M36" s="36" t="inlineStr">
+        <is>
+          <t>Diagrama de componentes con puertos, comunicación y bases de datos en docs/arquitectura/arquitectura.png (Figura 1 del informe); modelo ER en docs/modelo-er.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="26.85" customHeight="1" s="21">
       <c r="A37" s="31" t="inlineStr">

</xml_diff>